<commit_message>
feat: implement disease statistical analysis backend modules and evaluation management frontend components - Fixed assigned label counting bug - Added consensus mode - Updated label management and label synchronization interface
</commit_message>
<xml_diff>
--- a/backend/data/llm_evaluation_dataset.xlsx
+++ b/backend/data/llm_evaluation_dataset.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,12 +441,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ca nghi bệnh sởi ở Khánh Hòa giảm hơn 90%, nhưng bác sĩ vẫn khuyến cáo những điều cần nhớ</t>
+          <t>Một bệnh nhi ở Thanh Hóa chết do viêm não Nhật Bản</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SKĐS - Số ca sốt phát ban nghi bệnh sởi trên địa bàn tỉnh Khánh Hòa giảm mạnh so với năm ngoái, nhưng bác sĩ vẫn khuyến cáo người dân không được chủ quan.</t>
+          <t>Ngày 7-5, nguồn tin từ Trung tâm Kiểm soát bệnh tật tỉnh Thanh Hóa cho biết vừa ghi nhận một bệnh nhi chết do viêm não Nhật Bản. Bệnh nhi 14 tuổi, trú tại phường Đông Sơn.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -456,19 +456,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Xuất hiện thêm ổ dịch sốt xuất huyết, Hà Tĩnh tăng tốc phòng chống</t>
+          <t>Bão cytokine đẩy bé trai mắc tay chân miệng vào cửa tử</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SKĐS - Sau khi phát hiện ổ dịch, ngành Y tế Hà Tĩnh triển khai các biện pháp phòng, chống, phun hóa chất trong bán kính 200m nhằm ngăn chặn nguy cơ bùng phát dịch trên diện rộng.</t>
+          <t>Quảng Ninh Bé trai 4 tuổi nhập viện trong tình trạng sốt cao, nôn, thở gấp, bác sĩ phát hiện mắc tay chân miệng mức độ nặng nhất.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -478,19 +478,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>relevant</t>
+          <t>noise</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Bé gái 14 tuổi tử vong do viêm não Nhật Bản</t>
+          <t>Ca nghi bệnh sởi ở Khánh Hòa giảm hơn 90%, nhưng bác sĩ vẫn khuyến cáo những điều cần nhớ</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Thanh Hóa Bé gái 14 tuổi sốt cao, mệt mỏi, nói ngọng, suy đa tạng vì bệnh viêm não Nhật Bản, tử vong sau 5 ngày điều trị.</t>
+          <t>SKĐS - Số ca sốt phát ban nghi bệnh sởi trên địa bàn tỉnh Khánh Hòa giảm mạnh so với năm ngoái, nhưng bác sĩ vẫn khuyến cáo người dân không được chủ quan.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -500,19 +500,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>relevant</t>
+          <t>noise</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Hungary và EU bất đồng về giải ngân các khoản hỗ trợ hậu Covid-19</t>
+          <t>Xuất hiện thêm ổ dịch sốt xuất huyết, Hà Tĩnh tăng tốc phòng chống</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Trong vài ngày qua, các cuộc đàm phán với Liên minh châu Âu (EU) đã được đẩy mạnh để giải ngân khoản tiền 10,4 tỷ euro mà Hungary được hưởng theo quỹ phục hồi hậu đại dịch của EU. Số tiền này đã bị giữ lại do Hungary vi phạm luật EU dưới thời cựu thủ tướng Viktor Orbán với gần 16 năm cầm quyền và đã thất bại trong cuộc bầu cử vào tháng trước.</t>
+          <t>SKĐS - Sau khi phát hiện ổ dịch, ngành Y tế Hà Tĩnh triển khai các biện pháp phòng, chống, phun hóa chất trong bán kính 200m nhằm ngăn chặn nguy cơ bùng phát dịch trên diện rộng.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -522,19 +522,19 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Bão cytokine đẩy bé trai mắc tay chân miệng vào cửa tử</t>
+          <t>Bé gái 14 tuổi tử vong do viêm não Nhật Bản</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Quảng Ninh Bé trai 4 tuổi nhập viện trong tình trạng sốt cao, nôn, thở gấp, bác sĩ phát hiện mắc tay chân miệng mức độ nặng nhất.</t>
+          <t>Thanh Hóa Bé gái 14 tuổi sốt cao, mệt mỏi, nói ngọng, suy đa tạng vì bệnh viêm não Nhật Bản, tử vong sau 5 ngày điều trị.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -544,19 +544,19 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Một bệnh nhi ở Thanh Hóa chết do viêm não Nhật Bản</t>
+          <t>Hungary và EU bất đồng về giải ngân các khoản hỗ trợ hậu Covid-19</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Ngày 7-5, nguồn tin từ Trung tâm Kiểm soát bệnh tật tỉnh Thanh Hóa cho biết vừa ghi nhận một bệnh nhi chết do viêm não Nhật Bản. Bệnh nhi 14 tuổi, trú tại phường Đông Sơn.</t>
+          <t>Trong vài ngày qua, các cuộc đàm phán với Liên minh châu Âu (EU) đã được đẩy mạnh để giải ngân khoản tiền 10,4 tỷ euro mà Hungary được hưởng theo quỹ phục hồi hậu đại dịch của EU. Số tiền này đã bị giữ lại do Hungary vi phạm luật EU dưới thời cựu thủ tướng Viktor Orbán với gần 16 năm cầm quyền và đã thất bại trong cuộc bầu cử vào tháng trước.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -566,7 +566,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>relevant</t>
+          <t>noise</t>
         </is>
       </c>
     </row>
@@ -741,6 +741,2734 @@
         </is>
       </c>
       <c r="D15" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Nữ sinh tốt nghiệp xuất sắc, nhận học bổng Hàn Quốc sau một lần rẽ hướng</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SVO - Từng bắt đầu tại Đại học Kinh tế - ĐHQGHN, Ngân Hà (sinh viên ngành Truyền thông đa phương tiện, Đại học Thăng Long) lựa chọn rẽ hướng để tìm con đường phù hợp hơn. Từ những ngày học online vì dịch Covid-19 đến các dự án thực tế đầy áp lực, hành trình của cô là câu chuyện về sự kiên trì, thích nghi và trưởng thành qua từng lựa chọn.</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Hơn 18.000 ca 'tay chân miệng' ở phía Nam, chuyên gia nói gì về vắc xin mới?</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Vắc xin Envacgen vừa được Bộ Y tế cấp phép được kỳ vọng giúp giảm nguy cơ biến chứng nặng và tử vong do bệnh tay chân miệng.</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Phát hiện ổ dịch sốt xuất huyết thứ 2 tại phường Hoành Sơn, tỉnh Hà Tĩnh</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Theo thông tin từ Trung tâm Kiểm soát bệnh tật (CDC) Hà Tĩnh, "bệnh nhân số 0" của ổ dịch này là một bé trai sinh năm 2017. Bệnh nhi khởi phát triệu chứng từ ngày 3/5 với các dấu hiệu điển hình: sốt cao liên tục, đau đầu, đau cơ và chán ăn.</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Vượt đường xa đưa con đi tiêm vaccine</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Nghe thông báo Đăk Lăk có hai ca mắc bệnh do não mô cầu trong gia đình, chị H’Loan Byă, dân tộc Ê Đê, xã M’Drắk vượt 70 km đưa hai con đi tiêm vaccine.</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Lo ngại dịch bệnh, nhiều gia đình vượt hàng chục km để đưa con đi tiêm phòng bệnh</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Hàng loạt bệnh truyền nhiễm đồng loạt gia tăng và diễn biến phức tạp, làm dấy lên nguy cơ “dịch chồng dịch”. Trước lo ngại bùng phát trong mùa mưa, nhu cầu tiêm vaccine trên cả nước tăng mạnh, đặc biệt tại khu vực Tây Nguyên, nơi nhiều gia đình vượt hàng chục km để đưa con đi tiêm phòng.</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Ngành hàng không Mỹ gặp khủng hoảng lớn do giá nhiên liệu tăng vọt</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Bộ Giao thông Vận tải Mỹ cho biết các hãng hàng không chở khách lớn của nước này đã chi hơn 5 tỷ USD cho nhiên liệu máy bay trong tháng 3, tăng 1,8 tỷ USD, tương đương 56%, so với tháng 2. Giá nhiên liệu máy bay trung bình trong tháng 3 lên tới 3,13 USD/gallon, tăng 74 cent, tương đương 31% so với tháng trước. Trong khi đó, lượng nhiên liệu tiêu thụ cũng tăng 20%.</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Thứ trưởng Nguyễn Thị Liên Hương tiếp, làm việc với đoàn công tác Nhóm phụ trách Quốc gia của Quỹ Toàn cầu</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SKĐS - Chiều 6/5, tại Bộ Y tế, PGS.TS Nguyễn Thị Liên Hương, Thứ trưởng Bộ Y tế, Chủ tịch Ban Điều phối quốc gia Quỹ Toàn cầu phòng, chống HIV, Lao và Sốt Rét (CCM) Việt Nam tiếp và làm việc với đoàn công tác thuộc Nhóm phụ trách Quốc gia của Quỹ Toàn cầu.</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Cứu sống trẻ sơ sinh có nhóm máu hiếm</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Sáng 6-5, Bệnh viện Nhi Trung ương thông tin về việc lần đầu tiên, bệnh viện phát hiện, điều trị cho một bệnh nhi mang nhóm máu rất hiếm - nhóm máu Jk(a-b-3). Sau gần 2 tuần điều trị tích cực, trẻ đã ổn định và được xuất viện.</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Ngắm trọn tuyến đường 10 làn xe xuyên cù lao Phố với kinh phí 1.500 tỷ đồng</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Tuyến đường trục trung tâm Biên Hòa với nhánh chính 10 làn xe xuyên cù lao Phố đang dần lộ diện, mở ra trục kết nối đến trung tâm hành chính của Đồng Nai.</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Bé trai 7 tuổi nhập viện nguy kịch sau hai ngày sốt, bạch cầu tăng 8 lần</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>SKĐS - Hai ngày sau khi xuất hiện các dấu hiệu bất thường như sốt, lừ đừ và nổi ban xuất huyết, một bé trai 7 tuổi tại TPHCM đã được xác định mắc bệnh não mô cầu với biến chứng nhiễm trùng huyết.</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>[Infographic] 5 khuyến cáo phòng bệnh virus Hanta</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>SKĐS - Virus Hanta là nhóm virus có thể gây bệnh nặng ở người, như hội chứng phổi do virus Hanta hoặc sốt xuất huyết kèm hội chứng suy thận. Bệnh có thể diễn biến nhanh, gây khó thở, suy hô hấp, tụt huyết áp và có thể tử vong.</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TP.HCM: Cứu sống bé trai 7 tuổi mắc não mô cầu</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Nam bệnh nhi (7 tuổi, ở phường Long Trường, TP.HCM) sốt, lừ đừ đến ngày thứ 2 thì nổi các ban xuất huyết tập trung ở chân. Sau khi được đưa đến bệnh viện, bệnh nhi được theo dõi não mô cầu, nhiễm trùng huyết.</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>TPHCM: Cứu sống bé 7 tuổi mắc não mô cầu nhóm B diễn tiến nhanh</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>SKĐS - Bệnh nhi 7 tuổi sốt, lừ đừ và phát ban ở chân được chẩn đoán mắc não mô cầu nhóm B được điều trị thành công sau hơn 1 tuần phát hiện bệnh.</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Não mô cầu tấn công trẻ nhỏ, cảnh báo nguy cơ tử vong nhanh</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>(NLĐO) - Các bác sĩ cảnh báo số ca mắc não mô cầu đang có xu hướng gia tăng, tập trung chủ yếu ở trẻ nhỏ dưới 5 tuổi và thanh thiếu niên.</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Bé trai mắc não mô cầu thoát chết nhờ phát hiện nốt ‘tử ban’ trên da</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>TPO - Không phải cơn sốt, mà chính những nốt “tử ban” xuất hiện trên da khiến gia đình cảnh giác và đưa bé đi cấp cứu. Quyết định kịp thời này giúp bệnh nhi được phát hiện mắc não mô cầu và điều trị thành công.</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Cứu sống bé trai ở TPHCM mắc bệnh não mô cầu</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Sau 2 ngày sốt và nổi ban, một bé trai ở TPHCM rơi vào nguy hiểm do mắc bệnh não mô cầu. Bệnh nhi được chuyển sang khu vực cách ly và điều trị tích cực nhiều ngày.</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Hơn 260 công nhân khám định kỳ, ghi nhận hơn 300 bệnh</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Hơn 260 công nhân khám sức khỏe tổng quát thì phát hiện hơn 300 loại bệnh khác nhau, tức trung bình mỗi người mắc hơn một loại bệnh, trong đó có lao, ca nghi ung thư, theo lãnh đạo Công đoàn TP HCM.</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Bộ Y tế thông tin về diễn biến dịch bệnh trong nước</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Theo Bộ Y tế, trong 4 tuần từ 18.3 - 18.4, cả nước ghi nhận 302 trường hợp mắc Covid-19, không có ca tử vong. Trong 4 tháng từ 14.12.2025 - 18.4.2026, cả nước ghi nhận 356 trường hợp mắc Covid-19, 1 ca tử vong. So với cùng kỳ năm 2025, số mắc Covid-19 cao hơn 4,4 lần (đến 18.4.2026).</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>6.400 người mắc sốt xuất huyết trong một tháng, đã có ca tử vong</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Báo cáo công tác y tế tháng 4 của Bộ Y tế cho biết, từ ngày 18/3 đến 18/4, cả nước ghi nhận 6.408 trường hợp mắc sốt xuất huyết, trong đó có 1 ca tử vong.</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Sốt xuất huyết, tay chân miệng, COVID-19 gia tăng</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Theo báo cáo của Bộ Y tế, tháng qua cả nước ghi nhận số ca mắc sốt xuất huyết, tay chân miệng, COVID-19 gia tăng rõ rệt.</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Cúm mùa đến sớm, nhiều ca nặng ở người bệnh nền và lưu ý khi "tự chẩn đoán" bằng AI</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Cúm năm nay tại khu vực phía bắc có dấu hiệu đến sớm hơn thường lệ. Dù diễn biến nhìn chung vẫn điển hình nhưng các ca nặng ở nhóm có bệnh lý nền vẫn cần theo dõi và can thiệp kịp thời.</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Sốt xuất huyết, tay chân miệng tăng trong tháng 4</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>(NLĐO) - Sốt xuất huyết, tay chân miệng và viêm màng não do não mô cầu gia tăng trong tháng 4, Bộ Y tế cảnh báo dịch bệnh có thể diễn biến phức tạp.</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Ổ dịch sốt xuất huyết tại Hà Tĩnh chưa được khống chế, nguy cơ lan rộng</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>SKĐS - Sau gần 1 tháng ghi nhận ca bệnh đầu tiên, ổ dịch sốt xuất huyết tại Hà Tĩnh vẫn chưa được khống chế, với số ca mắc tăng nhanh. Ngành y tế địa phương cảnh báo nguy cơ lan rộng nếu không kiểm soát triệt để các ổ bọ gậy trong cộng đồng.</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Gần 230 trẻ ở Bangladesh tử vong do bệnh sởi</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Bangladesh đã ghi nhận 227 trường hợp tử vong ở trẻ em kể từ tháng 3, khi nước này đối mặt một trong những đợt bùng phát bệnh sởi tồi tệ nhất trong nhiều thập niên, theo AFP.</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Chuyên gia y tế tại Đà Nẵng cảnh báo về diễn tiến khó lường của sốt xuất huyết Dengue</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Những ca sốt xuất huyết Dengue nặng tại Đà Nẵng trong thời gian qua cho thấy những diễn tiến khó lường của bệnh. Với những triệu chứng có thể chuyển biến nhanh, đòi hỏi cần phải được theo dõi sát sao và điều trị kịp thời.</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Kiểm tra toàn bộ cơ sở tiêm vắc xin dịch vụ sau vụ tử vong do viêm não mô cầu</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>TPO - Sở Y tế Cà Mau quyết định thành lập đoàn kiểm tra, giám sát công tác tiêm chủng tại các cơ sở dịch vụ trên toàn tỉnh, chấn chỉnh hoạt động quảng cáo trong tiêm chủng, sau khi tỉnh có 2 người mắc, trong đó 1 người tử vong do viêm não mô cầu.</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Viêm não mô cầu: Từ sốt nhẹ đến tử vong chỉ trong vài giờ</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Viêm não mô cầu: Từ sốt nhẹ đến tử vong chỉ trong vài giờ</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Nổi mẩn tưởng dị ứng thông thường, trẻ gặp nguy cơ tổn thương thận</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>TPO - Nhiều trẻ phải nhập viện điều trị và ảnh hưởng đến cơ quan nội tạng chỉ từ những dấu hiệu ban đầu tưởng chừng đơn giản như ngứa và nổi mẩn đã gióng lên hồi chuông cảnh báo về sự chủ quan của không ít phụ huynh trước các biểu hiện bất thường của con trẻ.</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Xuất hiện viêm não mô cầu, Đắk Lắk khẩn trương truy vết người tiếp xúc</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Phát hiện ca tử vong do viêm não mô cầu, CDC Đắk Lắk đã phối hợp cùng cơ sở y tế địa phương tổ chức khử khuẩn, cấp thuốc kháng sinh dự phòng cho người tiếp xúc gần để ngăn chặn nguy cơ bùng phát dịch.</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Viêm não mô cầu, 1 trẻ không qua khỏi</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2 chú cháu trú tại phường Tân An, tỉnh Đắk Lắk dương tính với bệnh não mô cầu. Bệnh nặng khiến đứa trẻ không qua khỏi, còn người chú đang được cách ly điều trị.</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Dịch bệnh tay chân miệng diễn biến phức tạp</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Cả nước ghi nhận hơn 34.000 ca mắc tính đến giữa tháng 4, trong đó có 8 trường hợp tử vong.</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Cháu tử vong do não mô cầu, chú ruột 40 tuổi cũng nhiễm bệnh</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>TPO - Sau khi một cháu bé tử vong do viêm não mô cầu, ngành y tế Đắk Lắk lấy mẫu xét nghiệm, phát hiện thêm người chú ruột của cháu cũng dương tính.</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Phát hiện 2 bệnh nhân mắc viêm não mô cầu ở Đắk Lắk, 1 trường hợp tử vong</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Ngày 27/4, Trung tâm Kiểm soát bệnh tật tỉnh Đắk Lắk cho biết, trên địa bàn tỉnh vừa ghi nhận 2 bệnh nhân mắc viêm não mô cầu , trong đó 1 trường hợp bệnh nhi đã tử vong.</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Bé 2 tuổi tử vong do viêm não mô cầu, người thân phải cách ly y tế</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Bé 2 tuổi tử vong do viêm não mô cầu, người thân phải cách ly y tế</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Đắk Lắk: Bé trai 2 tuổi tử vong do mắc viêm não mô cầu</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>(PLO)- Tỉnh Đắk Lắk vừa ghi nhận một trường hợp bệnh nhi tử vong do mắc viêm não mô cầu trong tình trạng thể tối cấp.</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Ghi nhận 2 ca mắc viêm não mô cầu, 1 trẻ tử vong</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>(NLĐO) - Hai ca mắc viêm não mô cầu vừa được ghi nhận tại Đắk Lắk, trong đó 1 trẻ nhỏ đã tử vong, gióng lên cảnh báo về nguy cơ của bệnh truyền nhiễm nguy hiểm.</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Mỹ trấn an vi rút Hanta không phải COVID-19</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Quyền giám đốc CDC của Mỹ trấn an vi rút Hanta không phải COVID-19, và những công dân trở về từ tàu du lịch có thể không cần thiết phải bị cách ly.</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Triệu chứng nhiễm virus Hanta dễ nhầm với các bệnh khác, làm gì để phòng ngừa?</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Tổ chức Y tế Thế giới (WHO) virus Hanta là loại virus lây truyền từ động vật sang người, thường lây nhiễm tự nhiên ở loài gặm nhấm và đôi khi lây sang người. Thuộc họ Hantaviridae trong bộ Bunyavirales, mỗi chủng thường gắn với một loài vật chủ riêng, nơi chúng tồn tại nhưng gần như không gây biểu hiện rõ rệt.</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Sẽ xây dựng cơ chế đãi ngộ đặc thù cho lực lượng y tế tại hải đảo</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>TPO - Chuyến công tác của Đoàn cán bộ Bộ Y tế tại Trường Sa (Khánh Hòa) còn là dịp ngành y tế khảo sát thực trạng hệ thống y tế cơ sở tại các điểm đảo thuộc đặc khu này.</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Sốt cao mùa hè, cảnh giác viêm não Nhật Bản</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Viêm não Nhật Bản thường tăng từ tháng 5 đến tháng 7, khởi đầu bằng sốt cao, đau đầu, nôn ói nên dễ bị nhầm với bệnh nhiễm trùng thông thường.</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Khởi động điều tra tình trạng mù lòa, suy giảm thị lực trên toàn quốc</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>TPO - Tỉ lệ mù lòa và suy giảm thị lực tại Việt Nam đang đứng trước nhiều thay đổi do già hóa dân số và sự gia tăng của các bệnh không lây nhiễm. Trong bối cảnh đó, Bộ Y tế lần đầu triển khai lại cuộc điều tra quy mô toàn quốc về mù lòa sau hơn 10 năm, nhằm cập nhật thực trạng bệnh mắt trong cộng đồng và làm căn cứ xây dựng chính sách chăm sóc mắt giai đoạn mới.</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Bé gái vượt cửa tử khi men gan tăng gấp 100 lần</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>TP HCM Rơi vào sốc sốt xuất huyết khiến men gan tăng vọt gấp 100 lần bình thường, bé gái 10 tuổi được bác sĩ Bệnh viện Nhi đồng 1 cứu sống ngoạn mục.</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Chuyên gia về hồi sức cảnh báo căn bệnh quen thuộc gây nguy kịch cho trẻ</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>(NLĐO) - Một bé gái 10 tuổi bị sốc sốt xuất huyết Dengue nặng, men gan tăng gấp 100 lần bình thường vừa được các bác sĩ Bệnh viện Nhi Đồng 1 cứu sống thành công</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Virus Hanta: WHO khuyến nghị toàn bộ hành khách cách ly 42 ngày</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Theo Thủ tướng Pháp Sebastien Lecornu, một trong năm hành khách người Pháp đã xuất hiện triệu chứng nhiễm virus Hanta trong chuyến bay hồi hương chiều 10/5. Ngoài ra, các chuyến bay đưa công dân Canada, Hà Lan, Thổ Nhĩ Kỳ, Anh, Ireland và Mỹ về nước cũng đang được thực hiện với các chuyến cuối cùng sẽ rời đi vào tối 11/5.</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Thủy đậu biến chứng nhiễm khuẩn huyết, bé gái 6 tuổi nguy kịch</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>SKĐS - Khoa Nhi, Bệnh viện Bệnh Nhiệt đới Trung ương đang tích cực điều trị cho một bệnh nhi (6 tuổi, ở Lai Châu) nhập viện trong tình trạng suy hô hấp nặng và nhiễm khuẩn huyết do biến chứng thủy đậu.</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Vaccine cúm mùa 2026 và sự biến đổi của virus cúm: Những thông tin cần biết</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Vaccine cúm mùa 2026 và sự biến đổi của virus cúm: Những thông tin cần biết</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Chung tay xây dựng hệ thống y tế bền vững</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Châu Âu đang nỗ lực hỗ trợ châu Phi mở rộng năng lực sản xuất vắc-xin, qua đó góp phần bảo đảm an ninh y tế.</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Tàu bùng phát vi rút Hanta sắp cập bến, WHO trấn an không phải 'COVID-19 thứ hai'</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Tổng giám đốc Tổ chức Y tế thế giới (WHO) trực tiếp có mặt tại Tenerife (Tây Ban Nha) để giám sát chiến dịch sơ tán gần 150 hành khách từ tàu du lịch bùng phát vi rút Hanta, đồng thời trấn an người dân trên đảo này về nguy cơ lây nhiễm.</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Không nên xem nhẹ thủy đậu, bác sĩ cảnh báo biến chứng nguy hiểm</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Nhiều phụ huynh vẫn xem thủy đậu là bệnh nhẹ, chủ yếu sợ để lại sẹo. Nhưng theo các chuyên gia truyền nhiễm, thực tế tại bệnh viện đang ghi nhận không ít trẻ biến chứng nặng như viêm phổi hoại tử, viêm não...</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Vắc xin có từ lâu, vì sao ca nhập viện do thủy đậu vẫn tăng?</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Dù đã có vắc xin từ lâu, thủy đậu vẫn nằm trong nhóm bệnh truyền nhiễm phổ biến với hàng chục nghìn ca mỗi năm.</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Lập quy hoạch chi tiết Trung tâm hành chính tỉnh Nghệ An</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>TPO - Sở Xây dựng Nghệ An vừa đề xuất UBND tỉnh tiếp tục giao đơn vị tổ chức lập quy hoạch chi tiết tỷ lệ 1/500 Khu trung tâm hành chính tỉnh tại phường Vinh Lộc và xã Đông Lộc, tạo cơ sở triển khai dự án có tổng mức đầu tư gần 5.700 tỷ đồng.</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Cứu sống bệnh nhân trẻ mang 'quả mìn nổ chậm' trong não</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>TPO - Đột ngột đau đầu dữ dội, nôn ói và mất thăng bằng, nam thanh niên 30 tuổi được đưa vào cấp cứu và phát hiện đồng thời khối dị dạng mạch máu não gây xuất huyết và hai túi phình động mạch não nguy hiểm.</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Nguy cơ lây lan virus Ebola xuyên biên giới</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Theo phóng viên TTXVN tại châu Phi, ngày 15/5, Trung tâm Kiểm soát và phòng ngừa dịch bệnh châu Phi (ACDC) cho biết, Uganda đã phát hiện một ca nhiễm virus Ebola nhập cảnh từ Cộng hòa Dân chủ (CHDC) Congo, làm dấy lên lo ngại nguy cơ lây lan dịch bệnh xuyên biên giới.</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Anime "Your Name." đưa những ký ức học trò đẹp nhất trở lại màn ảnh rộng</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>HHTO - Từng tạo nên cơn sốt toàn cầu vào năm 2016, “Your Name.” chuẩn bị tái xuất màn ảnh rộng Việt Nam, đưa khán giả gặp lại Taki và Mitsuha trong câu chuyện hoán đổi thân xác đầy kỳ diệu.</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Bộ Công Thương thúc tiến độ triển khai xăng E10</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>TPO - Chỉ còn khoảng nửa tháng trước thời điểm bắt buộc bán xăng sinh học E10 trên phạm vi toàn quốc, Bộ Công Thương yêu cầu các doanh nghiệp đầu mối và phân phối xăng dầu khẩn trương chuẩn bị nguồn hàng, hệ thống phối trộn và cơ sở vật chất để sẵn sàng triển khai đồng loạt từ ngày 1/6.</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Bệnh viện Phổi Bình Thuận nêu lý do xin miễn xử phạt sai sót đấu thầu thời điểm COVID-19</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>(NLĐO) - Bệnh viện Phổi Bình Thuận giải trình vi phạm thủ tục đấu thầu vật tư chống dịch và đề nghị miễn xử phạt do xảy ra trong bối cảnh khẩn cấp</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Khởi tố ca sĩ Quang Lập và chủ Công ty BH Media</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Cục Cảnh sát điều tra tội phạm về tham nhũng, kinh tế, buôn lậu (C03, Bộ Công an) vừa ra quyết định khởi tố 5 vụ án hình sự liên quan đến hành vi xâm phạm quyền tác giả, quyền liên quan xảy ra tại nhiều công ty truyền thông, đơn vị giải trí.</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Mỹ tuyên bố tiêu diệt phó chỉ huy toàn cầu của ISIS trong chiến dịch tại Nigeria</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Trong bài đăng trên mạng xã hội Truht social tối 15/5, Tổng thống Mỹ cho biết chiến dịch được thực hiện theo chỉ thị trực tiếp của ông và ca ngợi đây là “một nhiệm vụ được lên kế hoạch tỉ mỉ và rất phức tạp”.</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>VNVC tặng kho bảo quản vaccine chuẩn quốc tế cho đặc khu Côn Đảo</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Sáng 16-5, Hệ thống Trung tâm Tiêm chủng VNVC đã trao tặng đặc khu Côn Đảo (TPHCM) gói tài trợ hơn 10 tỷ đồng, gồm: tiêm miễn phí vaccine cúm cho toàn bộ quân và dân đảo trong 3 năm liên tiếp, tặng 1 kho lạnh bảo quản vaccine đạt chuẩn quốc tế và cam kết ưu tiên cung ứng đầy đủ các vaccine thế hệ mới.</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Tăng cường năng lực y tế dự phòng cho Đặc khu Côn Đảo</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Trong định hướng phát triển Đặc khu Côn Đảo, nâng cao năng lực y tế dự phòng được xác định là nhiệm vụ quan trọng nhằm bảo vệ sức khỏe cộng đồng và phát triển bền vững vùng biển đảo. Chương trình hỗ trợ vaccine và hạ tầng bảo quản hiện đại là bước đi cụ thể cho định hướng chuyển từ chữa bệnh sang chủ động phòng bệnh.</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>unsure</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Viêm gan B có gây rụng tóc?</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Tôi bị viêm gan B mạn tính, đang điều trị và theo dõi. Gần đây, tóc tôi rụng nhiều có phải do viêm gan B không? (Thanh Mai, Tây Ninh)</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Virus Hanta lây qua phân, nước tiểu chuột: Chuyên gia khuyến cáo người dân</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Phó Giáo sư, Tiến sĩ Trần Đắc Phu cho biết, virus Hanta có thể gây hội chứng sốt xuất huyết kèm suy thận hoặc suy tim phổi nguy hiểm. Dù Việt Nam chưa ghi nhận ổ dịch điển hình, ngành y tế vẫn tăng cường giám sát nguy cơ xâm nhập.</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Thời tiết diễn biến phức tạp, Hà Tĩnh chủ động ngăn dịch sốt xuất huyết</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>SKĐS - Thời tiết diễn biến thất thường, Hà Tĩnh đang ghi nhận hai ổ dịch sốt xuất huyết. Ngành y tế địa phương đang triển khai nhiều giải pháp nhằm khoanh vùng, xử lý ổ dịch, hạn chế nguy cơ lây lan diện rộng.</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Hà Tĩnh tăng cường giám sát, phòng chống bệnh do virus Hanta</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>SKĐS - Trước nguy cơ bệnh do virus Hanta xâm nhập và lây lan, ngành y tế Hà Tĩnh tăng cường giám sát, chủ động triển khai các biện pháp phòng chống.</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>CEO Nvidia gây sốt mạng xã hội với khoảnh khắc ăn mì trên đường phố Bắc Kinh</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>CEO Nvidia Jensen Huang gây chú ý khi xuất hiện bất ngờ tại một ngõ nhỏ Bắc Kinh, thoải mái thưởng thức mì và ẩm thực đường phố như một du khách bình thường.</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Vaccine sốt rét không cần bảo quản lạnh</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Các nhà nghiên cứu từ Đại học Griffith (Australia) vừa phát triển thành công vaccine sốt rét thế hệ mới không yêu cầu bảo quản lạnh. Đây là bước tiến quan trọng vì bệnh sốt rét hiện cướp đi sinh mạng của hơn 500.000 người mỗi năm trên thế giới, chủ yếu tại những quốc gia đang phát triển.</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Điều tra: Thịt bẩn luồn lách đến bữa ăn - Kỳ 3: Thịt heo chết vào lò lạp xưởng</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>(PLO)- Từ những bãi đất trống ven đường, hàng trăm ký thịt heo không rõ nguồn gốc được mua bán, giao dịch ngay giữa đường trong đêm khuya.</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Bệnh viện Phổi Bình Thuận giải trình về vi phạm đấu thầu trong phòng chống dịch</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>TPO - Liên quan việc bị xác định có vi phạm hành chính trong lĩnh vực kế hoạch và đầu tư về đấu thầu, Bệnh viện Phổi Bình Thuận đã có văn bản gửi Sở Tài chính tỉnh Lâm Đồng để giải trình nguyên nhân dẫn đến sai sót trong quá trình mua sắm phục vụ phòng, chống dịch COVID-19.</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Hà Nội: "Đi từng ngõ, gõ từng nhà" chặn dịch sắp vào cao điểm</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>(Dân trí) - Những năm gần đây, số ca mắc sốt xuất huyết có xu hướng gia tăng, với các ổ dịch không chỉ tập trung tại nội thành mà còn lan rộng ra ngoại thành.</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>unsure</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Bệnh viện Phổi Bình Thuận đề nghị miễn xử phạt do vi phạm thủ tục đấu thầu</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Ngày 15-5, Bệnh viện Phổi Bình Thuận cho biết đã có văn bản gửi Sở Tài chính tỉnh Lâm Đồng giải trình các sai sót trong đấu thầu mua sắm vật tư phòng, chống dịch Covid-19 giai đoạn 2020-2021; đồng thời đề nghị xem xét miễn xử phạt vi phạm hành chính do vụ việc xảy ra trong “tình thế cấp thiết” thời điểm dịch bệnh.</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Vaccine cúm gia cầm đầu tiên thử nghiệm trên người giai đoạn 3</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Thử nghiệm được tổ chức tại Anh và Mỹ, dự kiến có 4.000 người tham gia, là vaccine đầu tiên thử nghiệm lâm sàng giai đoạn 3 trên người.</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Bé trai 4 tuổi nổi kín mụn nước toàn thân sau khi mắc cùng lúc zona thần kinh và thủy đậu</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>SKĐS - Bé trai 4 tuổi nhập viện trong tình trạng đau rát vùng lưng, bụng kèm các mụn nước mọc thành chùm rồi nhanh chóng lan khắp cơ thể. Đặc biệt, các bác sĩ xác định trẻ mắc đồng thời zona thần kinh và thủy đậu – tình trạng cực hiếm gặp ở trẻ khỏe mạnh.</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Lan truyền nguy hiểm dùng nước tiểu chữa bệnh, bác sĩ sửng sốt, cảnh báo nóng</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Những chia sẻ nguy hiểm về việc dùng nước tiểu để tắm, rửa mặt hay thậm chí nhỏ mắt đang gây xôn xao mạng xã hội, nhưng lại được một số người ca ngợi như “bài thuốc tự nhiên” chữa bệnh.</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Virus &amp;apos;bị lãng quên&amp;apos; ở người lớn quay trở lại tấn công từ mũi đến phổi</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Virus RSV không chỉ là mối đe dọa với trẻ nhỏ mà còn âm thầm gây biến chứng nặng, thậm chí tử vong ở người cao tuổi và bệnh nền nhưng bị xem nhẹ.</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Tiết canh vịt khiến 31 người ngộ độc</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Hưng Yên 31 người nhập viện với dấu hiệu nôn mửa, đau bụng, tiêu chảy, sốt sau khi ăn món tiết canh vịt tại xã Quỳnh Phụ.</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Cặp cá voi kiếm ăn ở biển Đăk Lăk</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Hai con cá voi dài khoảng 7-10 m xuất hiện kiếm ăn gần đảo Cù Lao Mái Nhà, xã Ô Loan, thu hút người dân và du khách theo dõi, sáng 15/5.</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Nguy cơ cao nam giới bị nhiễm HIV do quan hệ tình dục đồng giới</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Đó là một trong những thông tin từ Trung tâm Kiểm soát bệnh tật thành phố Huế nêu ra tại hội nghị triển khai chương trình phòng, chống HIV/AIDS năm 2026.</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Cảnh báo nhiều bệnh truyền nhiễm cùng lúc tăng mạnh ở TPHCM</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>TPHCM đưa ra cảnh báo khi số ca sốt xuất huyết tăng hơn 70%, bệnh tay chân miệng tăng hơn 100% so với cùng kỳ năm ngoái. Đáng chú ý, cả hai bệnh truyền nhiễm đều ghi nhận ca tử vong.</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Ngoại trưởng Mỹ gây sốt với khoảnh khắc 'ngỡ ngàng' trong Đại lễ đường Nhân dân</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Ngoại trưởng Mỹ gây chú ý với khoảnh khắc tỏ ra ngỡ ngàng và nhiều lần chỉ tay lên trần nhà trong Đại lễ đường Nhân dân ở Bắc Kinh.</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Huế mở rộng xét nghiệm HIV, hướng tới chấm dứt dịch bệnh AIDS vào năm 2030</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>SKĐS - Ngành Y tế TP Huế đang tiếp tục củng cố hệ thống phòng, chống HIV/AIDS, mở rộng xét nghiệm và nâng cao chất lượng điều trị nhằm hướng tới mục tiêu chấm dứt dịch bệnh AIDS vào năm 2030.</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Điều tra: Thịt bẩn luồn lách đến bữa ăn - Kỳ 2: Đường đi của xe chở thịt heo chết lúc rạng sáng</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>(PLO)- Từ lò mổ chui, những túi thịt heo chết được chia nhỏ, vận chuyển bằng xe máy hoặc xe tải len lỏi vào một số cơ sở cung cấp suất ăn công nghiệp.</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Cập nhật ổ dịch vi rút Hanta</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Tính đến ngày 14.5, tổng cộng đã có 11 người nghi nhiễm hoặc nhiễm vi rút Hanta liên quan du thuyền MV Hondius mang cờ Hà Lan, trong đó có 3 trường hợp tử vong, theo Tổ chức Y tế thế giới (WHO). Hiện chưa ghi nhận ca lây nhiễm nào bên ngoài du thuyền này.</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Bộ Y tế thông tin về chủng virus Hanta đang được WHO cảnh báo</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>SKĐS - Sau khi Tổ chức Y tế thế giới ghi nhận chùm ca nhiễm virus Hanta chủng Andes trên tàu du lịch quốc tế với 3 trường hợp tử vong, Bộ Y tế Việt Nam đã phát đi cảnh báo giám sát dịch tễ và khuyến cáo người dân không hoang mang nhưng cần chủ động phòng bệnh lây từ chuột sang người.</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>TPHCM cảnh báo nguy cơ bùng phát nhiều bệnh truyền nhiễm mùa hè</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>TPO - Hơn 16.000 ca sốt xuất huyết cùng số ca tay chân miệng tăng hơn gấp đôi so với cùng kỳ năm ngoái đang khiến TPHCM bước vào giai đoạn cảnh giác cao độ với dịch bệnh truyền nhiễm mùa hè.</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Giám sát dịch bệnh ngay từ cửa khẩu và tại các cơ sở khám, chữa bệnh</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Theo thông tin từ các cơ quan chức năng, tính đến chiều 14/5, Việt Nam chưa phát hiện trường hợp nào nhiễm virus Hanta.</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Việt Nam chưa phát hiện trường hợp nào nhiễm virus Hanta</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>(PLO)- Người phát ngôn Bộ Ngoại giao cho biết, theo thông tin từ các cơ quan chức năng, cho đến nay tại Việt Nam chưa phát hiện trường hợp nào nhiễm virus Hanta.</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>TP.HCM cảnh báo bệnh sốt xuất huyết sẽ gia tăng</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>(PLO)- Số ca tay chân miệng và sốt xuất huyết tăng, đã có trường hợp tử vong. Ngành y tế khuyến cáo người dân chủ động phòng bệnh, không chủ quan khi có triệu chứng nghi ngờ.</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Nhiều người bị suy giảm thị lực hoặc mù mắt do chơi Pickleball</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>TPO - Sau cú va chạm với bóng khi chơi Pickleball, một người đàn ông 39 tuổi phải nhập viện trong tình trạng xuất huyết mắt, thị lực suy giảm nghiêm trọng, trong khi một trường hợp khác đã mất vĩnh viễn một bên mắt do vỡ nhãn cầu. Các bác sĩ cảnh báo chấn thương mắt liên quan đến Pickleball đang gia tăng và có thể để lại hậu quả nặng nề nếu người chơi chủ quan.</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Tỷ phú Elon Musk gây sốt với màn check-in ngẫu hứng trước Đại lễ đường Nhân dân</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Video lan truyền trên mạng cho thấy ông Musk đứng cùng nhiều lãnh đạo doanh nghiệp và quan chức Mỹ, trong đó có Bộ trưởng Quốc phòng Pete Hegseth và Giám đốc điều hành Apple Tim Cook. Trong lúc mọi người xếp hàng chụp ảnh lưu niệm trước Đại lễ đường Nhân dân, ông Musk bất ngờ giơ điện thoại lên, xoay chậm một vòng để ghi lại khung cảnh xung quanh.</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Hiếm gặp, bé trai 4 tuổi đồng thời mắc 2 bệnh do cùng 1 virus</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>TPO - Bé trai 4 tuổi nhập viện trong tình trạng đau rát nhiều ở vùng lưng và bụng bên phải. Tại đây xuất hiện các cụm mụn nước, bọng nước tập trung trên nền da đỏ với kích thước khoảng 10x20 cm.</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Điều gì khiến Hantavirus trở thành mối lo y tế dù ít gặp?</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>SKĐS - Virus Hanta là tác nhân có thể gây tổn thương phổi hoặc suy thận nghiêm trọng ở người, với tỷ lệ tử vong cao ở một số trường hợp nặng. Dù bệnh tương đối hiếm gặp, các chuyên gia vẫn cảnh báo cần chú ý nguy cơ lây nhiễm từ động vật gặm nhấm và môi trường sống xung quanh...</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Khánh Hòa đã ghi nhận 2.254 ca tay chân miệng, bác sĩ khuyến cáo điều cần nhớ để phòng bệnh</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>SKĐS - Thống kê từ đầu năm đến ngày 12/5, toàn tỉnh Khánh Hòa đã ghi nhận tổng cộng 2.254 ca tay chân miệng, trong đó có một số trường hợp nặng.</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Cúm dạ dày bùng phát trên du thuyền chở hơn 1.700 người</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Cúm dạ dày bùng phát trên du thuyền Ambition chở hơn 1.700 người, và đã có một cụ ông lớn tuổi qua đời trên tàu này vì đau tim, theo Reuters ngày 13.5.</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Nguy cơ Ebola lây lan xuyên biên giới tại châu Phi</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Theo Bộ Y tế Uganda, bệnh nhân là một người đàn ông Congo 59 tuổi, nhập viện tại Bệnh viện Hồi giáo Kibuli ngày 11/5 và tử vong ngày 14/5. Nhà chức trách Uganda xác định, đây là ca bệnh nhập cảnh từ Cộng hòa Dân chủ (CHDC) Congo và cho biết, hiện chưa ghi nhận ca lây nhiễm trong cộng đồng tại Uganda.</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Từ cơn sốt nhẹ đến giây phút sinh tử - 24 giờ mong manh của con trước bệnh do não mô cầu</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Bệnh do não mô cầu đe dọa tính mạng trẻ nếu không được phát hiện và điều trị kịp thời. Đáng lo ngại hơn, 4 nhóm huyết thanh A, C, Y, W gây bệnh đang lưu hành tại Việt Nam.</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Giám sát phòng tránh lây lan vi-rút Hanta</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Ngày 13/5, Cục Phòng bệnh (Bộ Y tế) cho biết: Theo Tổ chức Y tế Thế giới, tính đến ngày 8/5/2026, chùm ca bệnh do virus Hanta trên tàu MV Hondius đã ghi nhận tám trường hợp, trong đó ba người chết, đều được xác định là chủng vi-rút Andes (ANDV).</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Giảm nguy cơ lây bệnh lao trong cộng đồng</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Tại Việt Nam, thách thức từ lao kháng thuốc và định kiến xã hội vẫn đang là rào cản ngăn người bệnh điều trị bệnh lao tại cộng đồng. Để có thể đạt mục tiêu cơ bản chấm dứt dịch bệnh lao vào năm 2030, ngành y tế cần tăng cường khám sàng lọc, phát hiện sớm bệnh lao, từ đó nâng cao hiệu quả điều trị, nhất là giảm nguy cơ lây lan trong cộng đồng.</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Pháp phong tỏa tàu chở hơn 1.700 người sau ca tử vong nghi do nhiễm virus</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Pháp phong tỏa tàu chở hơn 1.700 người sau ca tử vong nghi do nhiễm virus</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Điều tra: Thịt bẩn luồn lách đến bữa ăn - Kỳ 1: Thâm nhập lò mổ heo chết</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>(PLO)- Từ những con heo chết, PV ghi nhận một lò mổ hoạt động xuyên đêm, nơi thịt được xẻ ra, đóng thùng và nhanh chóng đưa đi tiêu thụ.</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Bộ Y tế thông tin về chủng vi rút Hanta đang được WHO cảnh báo</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Trước các thông tin quốc tế liên quan đến chùm ca bệnh do vi rút Hanta ghi nhận trên tàu du lịch quốc tế MV Hondius, ngày 13-5, Cục Phòng bệnh Bộ Y tế có văn bản khẩn thông tin về tình hình dịch bệnh và khuyến cáo.</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Chùm ca nhiễm virus Hanta trên tàu du lịch: Bộ Y tế phát khuyến cáo khẩn</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>(NLĐO) - Chùm ca nhiễm virus Hanta trên tàu MV Hondius khiến 3 người tử vong, Bộ Y tế khuyến cáo người dân theo dõi sức khỏe, chủ động phòng chống chuột.</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Việt Nam chưa ghi nhận ca mắc virus Hanta</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Chiều 13-5, Cục Phòng bệnh (Bộ Y tế) có công văn khẩn gửi các đơn vị chức năng của Bộ Y tế cập nhật thông tin về chùm ca bệnh do virus Hanta gây ra trên tàu du lịch quốc tế MV Hondius khi đang trên hành trình từ Argentina tới Cape Verde (quốc đảo ngoài khơi Tây Phi).</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Khám sàng lọc lao cho người dân tại vùng cao</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Các bác sĩ Bệnh viện Phổi Trung ương vừa thực hiện gần 2.000 lượt khám sàng lọc lao cho người dân tại vùng cao, qua đó kịp thời phát hiện bệnh lao cũng như các bệnh lý khác để đưa vào điều trị, cũng như bảo vệ cộng đồng khỏi nguồn lây.</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Hantavirus dễ nhầm với cúm có thể chuyển nặng nhanh</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Một chùm ca nhiễm Hantavirus xuất hiện trên tàu du lịch quốc tế với 3 trường hợp tử vong đang khiến giới y tế toàn cầu lo ngại. Bệnh có biểu hiện ban đầu rất dễ nhầm với cúm.</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>3 người tử vong trên tàu du lịch Hà Lan, Bộ Y tế khuyến cáo phòng bệnh từ chuột</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Trước thông tin về chùm ca bệnh do virus Hanta trên tàu du lịch Hà Lan, Cục Phòng bệnh (Bộ Y tế)  khuyến cáo người dân chủ động phòng bệnh, đặc biệt trong bối cảnh chuột phổ biến tại nhiều địa phương.</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Phòng, chống virus Hanta: Việt Nam tăng cường giám sát tại cửa khẩu, cơ sở khám bệnh, chữa bệnh</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Bộ Y tế cho biết, hiện chưa ghi nhận công dân Việt Nam có liên quan đến chùm ca bệnh nhiễm virus Hanta. Cục Phòng bệnh đã có văn bản đề nghị các địa phương tăng cường giám sát tại cửa khẩu, giám sát tại cơ sở khám bệnh, chữa bệnh.</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>3 người tử vong vì virus Hanta trên tàu du lịch, Việt Nam có nguy cơ?</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>3 người tử vong vì virus Hanta trên tàu du lịch, Việt Nam có nguy cơ?</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Phân biệt virus Hanta với cúm thường: Khi nào cần đi viện gấp?</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>SKĐS - Virus Hanta đang gây chú ý sau chùm ca bệnh nghiêm trọng trên tàu du lịch quốc tế năm 2026. Bệnh lây ra sao, triệu chứng thế nào và Việt Nam có nguy cơ không?</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Cách ly 42 ngày với người nguy cơ cao nhiễm virus Hanta</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Với người tiếp xúc nguy cơ cao nhiễm virus Hanta, Tổ chức Y tế thế giới WHO khuyến cáo theo dõi chủ động và cách ly 42 ngày.</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>WHO cảnh báo chùm ca virus Hanta gây tử vong, Việt Nam tăng cường giám sát</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Cục Phòng bệnh (Bộ Y tế) vừa phát công văn khẩn về bệnh do virus Hanta gây ra sau khi WHO ghi nhận chùm 11 ca bệnh trên tàu MV Hondius, trong đó có 3 ca tử vong.</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Sốc sốt xuất huyết, bệnh nhi 10 tuổi suy đa cơ quan, tổn thương gan cấp tính nguy kịch</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>SKĐS - Mới đây, Bệnh viện Nhi đồng 1 đã tiếp nhận và điều trị thành công cho một bé gái 10 tuổi mắc sốc sốt xuất huyết Dengue nặng, tổn thương gan cấp tính.</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Bệnh viện Hà Lan cách ly 12 nhân viên sau sự cố virus Hanta</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Bệnh viện Hà Lan cách ly 12 nhân viên sau sự cố virus Hanta</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Nhiều nước ghi nhận ca nhiễm virus Hanta liên quan tàu MV Hondius</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Nhiều nước ghi nhận ca nhiễm virus Hanta liên quan tàu MV Hondius</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Biến chứng thủy đậu, bé trai 6 tuổi nhiễm khuẩn huyết, phải thở máy nguy kịch</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>SKĐS - Tin từ Bệnh viện Bệnh Nhiệt đới Trung ương, khoa Nhi của bệnh viện đang điều trị cho bệnh nhi 6 tuổi trong tình trạng rất nặng sau biến chứng thủy đậu.</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Vaccine cúm mùa 2026 và sự biến đổi của virus cúm: Những thông tin cần biết</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Diễn biến phức tạp của virus cúm trong thời gian cuối năm 2025, đầu năm 2026 đang đặt ra yêu cầu cấp thiết về phòng bệnh chủ động. Các chuyên gia nhấn mạnh, tiêm vaccine cúm là giải pháp hiệu quả giúp giảm thiểu nguy cơ mắc bệnh cũng như các biến chứng nghiêm trọng.</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Manh mối dịch tễ về "bệnh nhân số 0" trong ổ dịch Hanta ở du thuyền hạng sang</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Theo New York Post, "bệnh nhân số 0" trong vụ bùng phát virus Hanta trên tàu du lịch đã được xác định là nhà điểu học người Hà Lan Leo Schilperoord (70 tuổi). Ông và vợ là bà Mirjam Schilperoord (69 tuổi) đều là những gương mặt quen thuộc trong cộng đồng nghiên cứu chim tại châu Âu.</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Một phụ nữ nhiễm bệnh nguy kịch, Pháp siết chặt kiểm soát virus Hanta</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Tổng thống Pháp Emmanuel Macron ngày 12/5 khẳng định tình hình liên quan đến virus Hanta tại Pháp vẫn “nằm trong tầm kiểm soát” của chính phủ, trong bối cảnh một phụ nữ Pháp nhiễm bệnh đang trong tình trạng nguy kịch và nhiều nước châu Âu tăng cường các biện pháp phòng dịch.</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Du thuyền có khách nhiễm vi rút Hanta hoàn tất sơ tán</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Reuters ngày 12.5 dẫn thông báo của nhà điều hành Oceanwide Expeditions (Hà Lan) cho hay du thuyền MV Hondius đã khởi hành từ Tây Ban Nha về Hà Lan với 25 thành viên thủy thủ đoàn cùng 1 bác sĩ và 1 điều dưỡng. Tất cả hành khách đã được sơ tán sau khi ổ dịch vi rút Hanta bùng phát trên du thuyền.</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Ukraine nêu điểm yếu khiến nhiều robot thất thế ngay lần đầu xung trận</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Ukraine nêu điểm yếu khiến nhiều robot thất thế ngay lần đầu xung trận</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Sơ tán sau 3 ca tử vong vì vi rút Hanta, tàu MV Hondius lên đường về Hà Lan</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Tàu MV Hondius rời Tây Ban Nha, hướng về Hà Lan. Một số hành khách tiếp tục có kết quả dương tính với vi rút Hanta sau khi hồi hương.</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Hà Lan cách ly 12 nhân viên y tế sau sự cố xử lý ca nhiễm virus Hanta</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Vụ việc xảy ra tại bệnh viện Radboudumc ở thành phố Nijmegen, nơi tiếp nhận một hành khách từ tàu du lịch MV Hondius vào ngày 7/5. Theo thông báo của bệnh viện, máu và nước tiểu của bệnh nhân đã được xử lý mà không thực hiện đầy đủ các quy trình an toàn nghiêm ngặt, dẫn đến việc 12 nhân viên y tế phải cách ly phòng ngừa trong thời gian 6 tuần.</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Vận hành nguồn Quỹ Toàn cầu công khai, minh bạch, đúng quy định và vì lợi ích của người dân</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>SKĐS - Chiều 12/5, tại Bộ Y tế, PGS.TS Nguyễn Thị Liên Hương, Thứ trưởng Bộ Y tế, Chủ tịch Ban điều phối Quốc gia Quỹ Toàn cầu phòng, chống AIDS, Lao và Sốt rét tại Việt Nam (CCM) chủ trì cuộc họp chuẩn bị xây dựng Hồ sơ đề xuất viện trợ Quỹ Toàn cầu, giai đoạn 2027-2029.</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Thái Lan siết chặt kiểm tra y tế tại sân bay quốc tế để ngăn chặn virus Hanta</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Cục trưởng DDC, Tiến sĩ Montien Kanasawadse, cho biết quyết định tăng cường quy trình sàng lọc sức khỏe đối với hành khách nhập cảnh từ các quốc gia và vùng lãnh thổ Nam Mỹ tại các sân bay quốc tế lớn, vừa để trấn an công chúng, vừa khẳng định chính phủ đã triển khai đầy đủ các bước phòng ngừa cần thiết, dù đến nay chưa ghi nhận ca nhiễm virus Hanta nào tại Thái Lan. Ông Montien nhấn mạnh, động thái này cũng nhằm bảo đảm môi trường du lịch an toàn.</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Bé trai 6 tuổi nguy kịch vì biến chứng nặng từ thủy đậu</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>TPO - Từ những nốt phỏng nước tưởng chừng thông thường do thủy đậu, một bé trai 6 tuổi ở Lai Châu đã rơi vào tình trạng nguy kịch với suy hô hấp nặng, nhiễm khuẩn huyết do phế cầu và phải thở máy xâm nhập.</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
         <is>
           <t>relevant</t>
         </is>

</xml_diff>

<commit_message>
feat: enhanced AI evaluation system, Mailtrap SMTP integration, background summary jobs and improved admin UI - implement detailed scan statistics (noise, irrelevant, unsure count) in SchedulerConfig and ScanResult - add background AI Daily Summary job using APScheduler - implement auto severity calculation for events based on case count and date age - improve Article Query with specific DiseaseCase matching to reduce false positives - refine Evaluation Management UI with latest session metrics card and custom pagination - enhance AlertsPage, DashboardOverview and location mapper utilities
</commit_message>
<xml_diff>
--- a/backend/data/llm_evaluation_dataset.xlsx
+++ b/backend/data/llm_evaluation_dataset.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D139"/>
+  <dimension ref="A1:D202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,12 +463,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bão cytokine đẩy bé trai mắc tay chân miệng vào cửa tử</t>
+          <t>Xuất hiện thêm ổ dịch sốt xuất huyết, Hà Tĩnh tăng tốc phòng chống</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Quảng Ninh Bé trai 4 tuổi nhập viện trong tình trạng sốt cao, nôn, thở gấp, bác sĩ phát hiện mắc tay chân miệng mức độ nặng nhất.</t>
+          <t>SKĐS - Sau khi phát hiện ổ dịch, ngành Y tế Hà Tĩnh triển khai các biện pháp phòng, chống, phun hóa chất trong bán kính 200m nhằm ngăn chặn nguy cơ bùng phát dịch trên diện rộng.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -478,19 +478,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ca nghi bệnh sởi ở Khánh Hòa giảm hơn 90%, nhưng bác sĩ vẫn khuyến cáo những điều cần nhớ</t>
+          <t>Bé gái 14 tuổi tử vong do viêm não Nhật Bản</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SKĐS - Số ca sốt phát ban nghi bệnh sởi trên địa bàn tỉnh Khánh Hòa giảm mạnh so với năm ngoái, nhưng bác sĩ vẫn khuyến cáo người dân không được chủ quan.</t>
+          <t>Thanh Hóa Bé gái 14 tuổi sốt cao, mệt mỏi, nói ngọng, suy đa tạng vì bệnh viêm não Nhật Bản, tử vong sau 5 ngày điều trị.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -500,19 +500,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Xuất hiện thêm ổ dịch sốt xuất huyết, Hà Tĩnh tăng tốc phòng chống</t>
+          <t>TP.HCM phát hiện hơn 20.000 ca bệnh lao mỗi năm, đẩy mạnh sàng lọc qua khám sức khỏe định kỳ</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SKĐS - Sau khi phát hiện ổ dịch, ngành Y tế Hà Tĩnh triển khai các biện pháp phòng, chống, phun hóa chất trong bán kính 200m nhằm ngăn chặn nguy cơ bùng phát dịch trên diện rộng.</t>
+          <t>TP.HCM hiện là địa phương phát hiện nhiều bệnh nhân lao nhất cả nước, với 20.000 ca mỗi năm. Dự kiến trong năm 2026, TP sẽ triển khai sàng lọc bệnh lao gắn với khám sức khỏe định kỳ, các chương trình sức khỏe cộng đồng.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -529,12 +529,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Bé gái 14 tuổi tử vong do viêm não Nhật Bản</t>
+          <t>Bé gái 14 tuổi tại Thanh Hóa tử vong do viêm não Nhật Bản</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Thanh Hóa Bé gái 14 tuổi sốt cao, mệt mỏi, nói ngọng, suy đa tạng vì bệnh viêm não Nhật Bản, tử vong sau 5 ngày điều trị.</t>
+          <t>SKĐS - Thanh Hóa ghi nhận một bé gái 14 tuổi tử vong do viêm não Nhật Bản trong tình trạng chưa tiêm vaccine và diễn tiến bệnh nhanh.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -551,12 +551,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Hungary và EU bất đồng về giải ngân các khoản hỗ trợ hậu Covid-19</t>
+          <t>Số bệnh nhân lao tăng cao</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Trong vài ngày qua, các cuộc đàm phán với Liên minh châu Âu (EU) đã được đẩy mạnh để giải ngân khoản tiền 10,4 tỷ euro mà Hungary được hưởng theo quỹ phục hồi hậu đại dịch của EU. Số tiền này đã bị giữ lại do Hungary vi phạm luật EU dưới thời cựu thủ tướng Viktor Orbán với gần 16 năm cầm quyền và đã thất bại trong cuộc bầu cử vào tháng trước.</t>
+          <t>Bộ Y tế ghi nhận hơn 119.000 ca bệnh lao mới trong năm 2025, tăng gần 5% so với năm trước.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -566,19 +566,19 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TP.HCM phát hiện hơn 20.000 ca bệnh lao mỗi năm, đẩy mạnh sàng lọc qua khám sức khỏe định kỳ</t>
+          <t>Phát hiện virus corona mới ở Thái Lan có khả năng lây sang người</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>TP.HCM hiện là địa phương phát hiện nhiều bệnh nhân lao nhất cả nước, với 20.000 ca mỗi năm. Dự kiến trong năm 2026, TP sẽ triển khai sàng lọc bệnh lao gắn với khám sức khỏe định kỳ, các chương trình sức khỏe cộng đồng.</t>
+          <t>Một nhóm nhà khoa học Nhật Bản và Thái Lan thông báo một loại virus corona mới có liên quan đến loại gây ra đại dịch Covid-19 đã được phát hiện ở Thái Lan, và nó có khả năng lây nhiễm sang người.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -595,12 +595,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Phân biệt triệu chứng do virus Hanta với các bệnh truyền nhiễm khác</t>
+          <t>Phát hiện ổ dịch sốt xuất huyết thứ 2 tại phường Hoành Sơn, tỉnh Hà Tĩnh</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Triệu chứng bệnh do virus Hanta từ chuột dễ nhầm với cúm, sốt xuất huyết hay sốt siêu vi, song khác ở chỗ đi tiểu ít, phù mặt hoặc chân, tụt huyết áp, khó thở sau 3-5 ngày.</t>
+          <t>Theo thông tin từ Trung tâm Kiểm soát bệnh tật (CDC) Hà Tĩnh, "bệnh nhân số 0" của ổ dịch này là một bé trai sinh năm 2017. Bệnh nhi khởi phát triệu chứng từ ngày 3/5 với các dấu hiệu điển hình: sốt cao liên tục, đau đầu, đau cơ và chán ăn.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -610,19 +610,19 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Chồng mắc viêm gan B, làm sao để tránh lây bệnh?</t>
+          <t>TP.HCM: Cứu sống bé trai 7 tuổi mắc não mô cầu</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Chồng vừa mới phát hiện mắc bệnh viêm gan B, tôi làm cách nào để phòng lây nhiễm? (Như Giang, 38 tuổi, Đăk Lăk)</t>
+          <t>Nam bệnh nhi (7 tuổi, ở phường Long Trường, TP.HCM) sốt, lừ đừ đến ngày thứ 2 thì nổi các ban xuất huyết tập trung ở chân. Sau khi được đưa đến bệnh viện, bệnh nhi được theo dõi não mô cầu, nhiễm trùng huyết.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -632,19 +632,19 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Bé gái 14 tuổi tại Thanh Hóa tử vong do viêm não Nhật Bản</t>
+          <t>TPHCM: Cứu sống bé 7 tuổi mắc não mô cầu nhóm B diễn tiến nhanh</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>SKĐS - Thanh Hóa ghi nhận một bé gái 14 tuổi tử vong do viêm não Nhật Bản trong tình trạng chưa tiêm vaccine và diễn tiến bệnh nhanh.</t>
+          <t>SKĐS - Bệnh nhi 7 tuổi sốt, lừ đừ và phát ban ở chân được chẩn đoán mắc não mô cầu nhóm B được điều trị thành công sau hơn 1 tuần phát hiện bệnh.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -661,12 +661,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Số bệnh nhân lao tăng cao</t>
+          <t>Não mô cầu tấn công trẻ nhỏ, cảnh báo nguy cơ tử vong nhanh</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Bộ Y tế ghi nhận hơn 119.000 ca bệnh lao mới trong năm 2025, tăng gần 5% so với năm trước.</t>
+          <t>(NLĐO) - Các bác sĩ cảnh báo số ca mắc não mô cầu đang có xu hướng gia tăng, tập trung chủ yếu ở trẻ nhỏ dưới 5 tuổi và thanh thiếu niên.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -683,12 +683,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Cơn bão cytokine đẩy bé 4 tuổi mắc tay chân miệng vào nguy kịch</t>
+          <t>6.400 người mắc sốt xuất huyết trong một tháng, đã có ca tử vong</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Sau 3 ngày sốt từng cơn kèm nhiều dấu hiệu xấu, bé trai 4 tuổi vào viện được xác định mắc tay chân miệng độ 4 rồi diễn biến xấu rất nhanh, nguy cơ tử vong cao.</t>
+          <t>Báo cáo công tác y tế tháng 4 của Bộ Y tế cho biết, từ ngày 18/3 đến 18/4, cả nước ghi nhận 6.408 trường hợp mắc sốt xuất huyết, trong đó có 1 ca tử vong.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -698,19 +698,19 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Còn 40% ca lao ngoài cộng đồng: Khám sức khỏe định kỳ mở 'cánh cửa' phát hiện sớm bệnh lao</t>
+          <t>Sốt xuất huyết, tay chân miệng, COVID-19 gia tăng</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>SKĐS - Theo WHO, bệnh lao vẫn là một trong những bệnh truyền nhiễm nguy hiểm nhất thế giới khi mỗi ngày có hơn 3.400 người tử vong và gần 30.000 ca mắc mới. Tại Việt Nam, dù công tác phòng chống lao đạt nhiều kết quả tích cực, ngành y tế vẫn đối mặt thực trạng đáng lo ngại: khoảng 40% người mắc lao chưa được phát hiện.</t>
+          <t>Theo báo cáo của Bộ Y tế, tháng qua cả nước ghi nhận số ca mắc sốt xuất huyết, tay chân miệng, COVID-19 gia tăng rõ rệt.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -720,19 +720,19 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Phát hiện virus corona mới ở Thái Lan có khả năng lây sang người</t>
+          <t>Cúm mùa đến sớm, nhiều ca nặng ở người bệnh nền và lưu ý khi "tự chẩn đoán" bằng AI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Một nhóm nhà khoa học Nhật Bản và Thái Lan thông báo một loại virus corona mới có liên quan đến loại gây ra đại dịch Covid-19 đã được phát hiện ở Thái Lan, và nó có khả năng lây nhiễm sang người.</t>
+          <t>Cúm năm nay tại khu vực phía bắc có dấu hiệu đến sớm hơn thường lệ. Dù diễn biến nhìn chung vẫn điển hình nhưng các ca nặng ở nhóm có bệnh lý nền vẫn cần theo dõi và can thiệp kịp thời.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -749,12 +749,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Nữ sinh tốt nghiệp xuất sắc, nhận học bổng Hàn Quốc sau một lần rẽ hướng</t>
+          <t>Sốt xuất huyết, tay chân miệng tăng trong tháng 4</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>SVO - Từng bắt đầu tại Đại học Kinh tế - ĐHQGHN, Ngân Hà (sinh viên ngành Truyền thông đa phương tiện, Đại học Thăng Long) lựa chọn rẽ hướng để tìm con đường phù hợp hơn. Từ những ngày học online vì dịch Covid-19 đến các dự án thực tế đầy áp lực, hành trình của cô là câu chuyện về sự kiên trì, thích nghi và trưởng thành qua từng lựa chọn.</t>
+          <t>(NLĐO) - Sốt xuất huyết, tay chân miệng và viêm màng não do não mô cầu gia tăng trong tháng 4, Bộ Y tế cảnh báo dịch bệnh có thể diễn biến phức tạp.</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -764,19 +764,19 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Hơn 18.000 ca 'tay chân miệng' ở phía Nam, chuyên gia nói gì về vắc xin mới?</t>
+          <t>Ổ dịch sốt xuất huyết tại Hà Tĩnh chưa được khống chế, nguy cơ lan rộng</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Vắc xin Envacgen vừa được Bộ Y tế cấp phép được kỳ vọng giúp giảm nguy cơ biến chứng nặng và tử vong do bệnh tay chân miệng.</t>
+          <t>SKĐS - Sau gần 1 tháng ghi nhận ca bệnh đầu tiên, ổ dịch sốt xuất huyết tại Hà Tĩnh vẫn chưa được khống chế, với số ca mắc tăng nhanh. Ngành y tế địa phương cảnh báo nguy cơ lan rộng nếu không kiểm soát triệt để các ổ bọ gậy trong cộng đồng.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -786,19 +786,19 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Phát hiện ổ dịch sốt xuất huyết thứ 2 tại phường Hoành Sơn, tỉnh Hà Tĩnh</t>
+          <t>Gần 230 trẻ ở Bangladesh tử vong do bệnh sởi</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Theo thông tin từ Trung tâm Kiểm soát bệnh tật (CDC) Hà Tĩnh, "bệnh nhân số 0" của ổ dịch này là một bé trai sinh năm 2017. Bệnh nhi khởi phát triệu chứng từ ngày 3/5 với các dấu hiệu điển hình: sốt cao liên tục, đau đầu, đau cơ và chán ăn.</t>
+          <t>Bangladesh đã ghi nhận 227 trường hợp tử vong ở trẻ em kể từ tháng 3, khi nước này đối mặt một trong những đợt bùng phát bệnh sởi tồi tệ nhất trong nhiều thập niên, theo AFP.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -815,12 +815,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Vượt đường xa đưa con đi tiêm vaccine</t>
+          <t>Chuyên gia y tế tại Đà Nẵng cảnh báo về diễn tiến khó lường của sốt xuất huyết Dengue</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Nghe thông báo Đăk Lăk có hai ca mắc bệnh do não mô cầu trong gia đình, chị H’Loan Byă, dân tộc Ê Đê, xã M’Drắk vượt 70 km đưa hai con đi tiêm vaccine.</t>
+          <t>Những ca sốt xuất huyết Dengue nặng tại Đà Nẵng trong thời gian qua cho thấy những diễn tiến khó lường của bệnh. Với những triệu chứng có thể chuyển biến nhanh, đòi hỏi cần phải được theo dõi sát sao và điều trị kịp thời.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -830,19 +830,19 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Lo ngại dịch bệnh, nhiều gia đình vượt hàng chục km để đưa con đi tiêm phòng bệnh</t>
+          <t>Xuất hiện viêm não mô cầu, Đắk Lắk khẩn trương truy vết người tiếp xúc</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Hàng loạt bệnh truyền nhiễm đồng loạt gia tăng và diễn biến phức tạp, làm dấy lên nguy cơ “dịch chồng dịch”. Trước lo ngại bùng phát trong mùa mưa, nhu cầu tiêm vaccine trên cả nước tăng mạnh, đặc biệt tại khu vực Tây Nguyên, nơi nhiều gia đình vượt hàng chục km để đưa con đi tiêm phòng.</t>
+          <t>Phát hiện ca tử vong do viêm não mô cầu, CDC Đắk Lắk đã phối hợp cùng cơ sở y tế địa phương tổ chức khử khuẩn, cấp thuốc kháng sinh dự phòng cho người tiếp xúc gần để ngăn chặn nguy cơ bùng phát dịch.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -852,19 +852,19 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ngành hàng không Mỹ gặp khủng hoảng lớn do giá nhiên liệu tăng vọt</t>
+          <t>Viêm não mô cầu, 1 trẻ không qua khỏi</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Bộ Giao thông Vận tải Mỹ cho biết các hãng hàng không chở khách lớn của nước này đã chi hơn 5 tỷ USD cho nhiên liệu máy bay trong tháng 3, tăng 1,8 tỷ USD, tương đương 56%, so với tháng 2. Giá nhiên liệu máy bay trung bình trong tháng 3 lên tới 3,13 USD/gallon, tăng 74 cent, tương đương 31% so với tháng trước. Trong khi đó, lượng nhiên liệu tiêu thụ cũng tăng 20%.</t>
+          <t>2 chú cháu trú tại phường Tân An, tỉnh Đắk Lắk dương tính với bệnh não mô cầu. Bệnh nặng khiến đứa trẻ không qua khỏi, còn người chú đang được cách ly điều trị.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -874,19 +874,19 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Thứ trưởng Nguyễn Thị Liên Hương tiếp, làm việc với đoàn công tác Nhóm phụ trách Quốc gia của Quỹ Toàn cầu</t>
+          <t>Dịch bệnh tay chân miệng diễn biến phức tạp</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SKĐS - Chiều 6/5, tại Bộ Y tế, PGS.TS Nguyễn Thị Liên Hương, Thứ trưởng Bộ Y tế, Chủ tịch Ban Điều phối quốc gia Quỹ Toàn cầu phòng, chống HIV, Lao và Sốt Rét (CCM) Việt Nam tiếp và làm việc với đoàn công tác thuộc Nhóm phụ trách Quốc gia của Quỹ Toàn cầu.</t>
+          <t>Cả nước ghi nhận hơn 34.000 ca mắc tính đến giữa tháng 4, trong đó có 8 trường hợp tử vong.</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -896,19 +896,19 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Cứu sống trẻ sơ sinh có nhóm máu hiếm</t>
+          <t>Phát hiện 2 bệnh nhân mắc viêm não mô cầu ở Đắk Lắk, 1 trường hợp tử vong</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Sáng 6-5, Bệnh viện Nhi Trung ương thông tin về việc lần đầu tiên, bệnh viện phát hiện, điều trị cho một bệnh nhi mang nhóm máu rất hiếm - nhóm máu Jk(a-b-3). Sau gần 2 tuần điều trị tích cực, trẻ đã ổn định và được xuất viện.</t>
+          <t>Ngày 27/4, Trung tâm Kiểm soát bệnh tật tỉnh Đắk Lắk cho biết, trên địa bàn tỉnh vừa ghi nhận 2 bệnh nhân mắc viêm não mô cầu , trong đó 1 trường hợp bệnh nhi đã tử vong.</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -918,19 +918,19 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ngắm trọn tuyến đường 10 làn xe xuyên cù lao Phố với kinh phí 1.500 tỷ đồng</t>
+          <t>Đắk Lắk: Bé trai 2 tuổi tử vong do mắc viêm não mô cầu</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Tuyến đường trục trung tâm Biên Hòa với nhánh chính 10 làn xe xuyên cù lao Phố đang dần lộ diện, mở ra trục kết nối đến trung tâm hành chính của Đồng Nai.</t>
+          <t>(PLO)- Tỉnh Đắk Lắk vừa ghi nhận một trường hợp bệnh nhi tử vong do mắc viêm não mô cầu trong tình trạng thể tối cấp.</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -940,19 +940,19 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Bé trai 7 tuổi nhập viện nguy kịch sau hai ngày sốt, bạch cầu tăng 8 lần</t>
+          <t>Ghi nhận 2 ca mắc viêm não mô cầu, 1 trẻ tử vong</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>SKĐS - Hai ngày sau khi xuất hiện các dấu hiệu bất thường như sốt, lừ đừ và nổi ban xuất huyết, một bé trai 7 tuổi tại TPHCM đã được xác định mắc bệnh não mô cầu với biến chứng nhiễm trùng huyết.</t>
+          <t>(NLĐO) - Hai ca mắc viêm não mô cầu vừa được ghi nhận tại Đắk Lắk, trong đó 1 trẻ nhỏ đã tử vong, gióng lên cảnh báo về nguy cơ của bệnh truyền nhiễm nguy hiểm.</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -962,19 +962,19 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>[Infographic] 5 khuyến cáo phòng bệnh virus Hanta</t>
+          <t>Sốt cao mùa hè, cảnh giác viêm não Nhật Bản</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>SKĐS - Virus Hanta là nhóm virus có thể gây bệnh nặng ở người, như hội chứng phổi do virus Hanta hoặc sốt xuất huyết kèm hội chứng suy thận. Bệnh có thể diễn biến nhanh, gây khó thở, suy hô hấp, tụt huyết áp và có thể tử vong.</t>
+          <t>Viêm não Nhật Bản thường tăng từ tháng 5 đến tháng 7, khởi đầu bằng sốt cao, đau đầu, nôn ói nên dễ bị nhầm với bệnh nhiễm trùng thông thường.</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -984,19 +984,19 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TP.HCM: Cứu sống bé trai 7 tuổi mắc não mô cầu</t>
+          <t>Bé gái vượt cửa tử khi men gan tăng gấp 100 lần</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Nam bệnh nhi (7 tuổi, ở phường Long Trường, TP.HCM) sốt, lừ đừ đến ngày thứ 2 thì nổi các ban xuất huyết tập trung ở chân. Sau khi được đưa đến bệnh viện, bệnh nhi được theo dõi não mô cầu, nhiễm trùng huyết.</t>
+          <t>TP HCM Rơi vào sốc sốt xuất huyết khiến men gan tăng vọt gấp 100 lần bình thường, bé gái 10 tuổi được bác sĩ Bệnh viện Nhi đồng 1 cứu sống ngoạn mục.</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1013,12 +1013,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>TPHCM: Cứu sống bé 7 tuổi mắc não mô cầu nhóm B diễn tiến nhanh</t>
+          <t>Chuyên gia về hồi sức cảnh báo căn bệnh quen thuộc gây nguy kịch cho trẻ</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>SKĐS - Bệnh nhi 7 tuổi sốt, lừ đừ và phát ban ở chân được chẩn đoán mắc não mô cầu nhóm B được điều trị thành công sau hơn 1 tuần phát hiện bệnh.</t>
+          <t>(NLĐO) - Một bé gái 10 tuổi bị sốc sốt xuất huyết Dengue nặng, men gan tăng gấp 100 lần bình thường vừa được các bác sĩ Bệnh viện Nhi Đồng 1 cứu sống thành công</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1035,12 +1035,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Não mô cầu tấn công trẻ nhỏ, cảnh báo nguy cơ tử vong nhanh</t>
+          <t>Thủy đậu biến chứng nhiễm khuẩn huyết, bé gái 6 tuổi nguy kịch</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>(NLĐO) - Các bác sĩ cảnh báo số ca mắc não mô cầu đang có xu hướng gia tăng, tập trung chủ yếu ở trẻ nhỏ dưới 5 tuổi và thanh thiếu niên.</t>
+          <t>SKĐS - Khoa Nhi, Bệnh viện Bệnh Nhiệt đới Trung ương đang tích cực điều trị cho một bệnh nhi (6 tuổi, ở Lai Châu) nhập viện trong tình trạng suy hô hấp nặng và nhiễm khuẩn huyết do biến chứng thủy đậu.</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1057,12 +1057,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Bé trai mắc não mô cầu thoát chết nhờ phát hiện nốt ‘tử ban’ trên da</t>
+          <t>Không nên xem nhẹ thủy đậu, bác sĩ cảnh báo biến chứng nguy hiểm</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>TPO - Không phải cơn sốt, mà chính những nốt “tử ban” xuất hiện trên da khiến gia đình cảnh giác và đưa bé đi cấp cứu. Quyết định kịp thời này giúp bệnh nhi được phát hiện mắc não mô cầu và điều trị thành công.</t>
+          <t>Nhiều phụ huynh vẫn xem thủy đậu là bệnh nhẹ, chủ yếu sợ để lại sẹo. Nhưng theo các chuyên gia truyền nhiễm, thực tế tại bệnh viện đang ghi nhận không ít trẻ biến chứng nặng như viêm phổi hoại tử, viêm não...</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1072,19 +1072,19 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Cứu sống bé trai ở TPHCM mắc bệnh não mô cầu</t>
+          <t>Vắc xin có từ lâu, vì sao ca nhập viện do thủy đậu vẫn tăng?</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sau 2 ngày sốt và nổi ban, một bé trai ở TPHCM rơi vào nguy hiểm do mắc bệnh não mô cầu. Bệnh nhi được chuyển sang khu vực cách ly và điều trị tích cực nhiều ngày.</t>
+          <t>Dù đã có vắc xin từ lâu, thủy đậu vẫn nằm trong nhóm bệnh truyền nhiễm phổ biến với hàng chục nghìn ca mỗi năm.</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1094,19 +1094,19 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Hơn 260 công nhân khám định kỳ, ghi nhận hơn 300 bệnh</t>
+          <t>Nguy cơ lây lan virus Ebola xuyên biên giới</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Hơn 260 công nhân khám sức khỏe tổng quát thì phát hiện hơn 300 loại bệnh khác nhau, tức trung bình mỗi người mắc hơn một loại bệnh, trong đó có lao, ca nghi ung thư, theo lãnh đạo Công đoàn TP HCM.</t>
+          <t>Theo phóng viên TTXVN tại châu Phi, ngày 15/5, Trung tâm Kiểm soát và phòng ngừa dịch bệnh châu Phi (ACDC) cho biết, Uganda đã phát hiện một ca nhiễm virus Ebola nhập cảnh từ Cộng hòa Dân chủ (CHDC) Congo, làm dấy lên lo ngại nguy cơ lây lan dịch bệnh xuyên biên giới.</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1116,19 +1116,19 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Bộ Y tế thông tin về diễn biến dịch bệnh trong nước</t>
+          <t>Tăng cường năng lực y tế dự phòng cho Đặc khu Côn Đảo</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Theo Bộ Y tế, trong 4 tuần từ 18.3 - 18.4, cả nước ghi nhận 302 trường hợp mắc Covid-19, không có ca tử vong. Trong 4 tháng từ 14.12.2025 - 18.4.2026, cả nước ghi nhận 356 trường hợp mắc Covid-19, 1 ca tử vong. So với cùng kỳ năm 2025, số mắc Covid-19 cao hơn 4,4 lần (đến 18.4.2026).</t>
+          <t>Trong định hướng phát triển Đặc khu Côn Đảo, nâng cao năng lực y tế dự phòng được xác định là nhiệm vụ quan trọng nhằm bảo vệ sức khỏe cộng đồng và phát triển bền vững vùng biển đảo. Chương trình hỗ trợ vaccine và hạ tầng bảo quản hiện đại là bước đi cụ thể cho định hướng chuyển từ chữa bệnh sang chủ động phòng bệnh.</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1138,19 +1138,19 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>unsure</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>6.400 người mắc sốt xuất huyết trong một tháng, đã có ca tử vong</t>
+          <t>Virus Hanta lây qua phân, nước tiểu chuột: Chuyên gia khuyến cáo người dân</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Báo cáo công tác y tế tháng 4 của Bộ Y tế cho biết, từ ngày 18/3 đến 18/4, cả nước ghi nhận 6.408 trường hợp mắc sốt xuất huyết, trong đó có 1 ca tử vong.</t>
+          <t>Phó Giáo sư, Tiến sĩ Trần Đắc Phu cho biết, virus Hanta có thể gây hội chứng sốt xuất huyết kèm suy thận hoặc suy tim phổi nguy hiểm. Dù Việt Nam chưa ghi nhận ổ dịch điển hình, ngành y tế vẫn tăng cường giám sát nguy cơ xâm nhập.</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1167,12 +1167,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Sốt xuất huyết, tay chân miệng, COVID-19 gia tăng</t>
+          <t>Thời tiết diễn biến phức tạp, Hà Tĩnh chủ động ngăn dịch sốt xuất huyết</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Theo báo cáo của Bộ Y tế, tháng qua cả nước ghi nhận số ca mắc sốt xuất huyết, tay chân miệng, COVID-19 gia tăng rõ rệt.</t>
+          <t>SKĐS - Thời tiết diễn biến thất thường, Hà Tĩnh đang ghi nhận hai ổ dịch sốt xuất huyết. Ngành y tế địa phương đang triển khai nhiều giải pháp nhằm khoanh vùng, xử lý ổ dịch, hạn chế nguy cơ lây lan diện rộng.</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1189,12 +1189,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Cúm mùa đến sớm, nhiều ca nặng ở người bệnh nền và lưu ý khi "tự chẩn đoán" bằng AI</t>
+          <t>Hà Tĩnh tăng cường giám sát, phòng chống bệnh do virus Hanta</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Cúm năm nay tại khu vực phía bắc có dấu hiệu đến sớm hơn thường lệ. Dù diễn biến nhìn chung vẫn điển hình nhưng các ca nặng ở nhóm có bệnh lý nền vẫn cần theo dõi và can thiệp kịp thời.</t>
+          <t>SKĐS - Trước nguy cơ bệnh do virus Hanta xâm nhập và lây lan, ngành y tế Hà Tĩnh tăng cường giám sát, chủ động triển khai các biện pháp phòng chống.</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1211,12 +1211,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Sốt xuất huyết, tay chân miệng tăng trong tháng 4</t>
+          <t>Hà Nội: "Đi từng ngõ, gõ từng nhà" chặn dịch sắp vào cao điểm</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>(NLĐO) - Sốt xuất huyết, tay chân miệng và viêm màng não do não mô cầu gia tăng trong tháng 4, Bộ Y tế cảnh báo dịch bệnh có thể diễn biến phức tạp.</t>
+          <t>(Dân trí) - Những năm gần đây, số ca mắc sốt xuất huyết có xu hướng gia tăng, với các ổ dịch không chỉ tập trung tại nội thành mà còn lan rộng ra ngoại thành.</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1226,19 +1226,19 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>relevant</t>
+          <t>unsure</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Ổ dịch sốt xuất huyết tại Hà Tĩnh chưa được khống chế, nguy cơ lan rộng</t>
+          <t>Vaccine cúm gia cầm đầu tiên thử nghiệm trên người giai đoạn 3</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>SKĐS - Sau gần 1 tháng ghi nhận ca bệnh đầu tiên, ổ dịch sốt xuất huyết tại Hà Tĩnh vẫn chưa được khống chế, với số ca mắc tăng nhanh. Ngành y tế địa phương cảnh báo nguy cơ lan rộng nếu không kiểm soát triệt để các ổ bọ gậy trong cộng đồng.</t>
+          <t>Thử nghiệm được tổ chức tại Anh và Mỹ, dự kiến có 4.000 người tham gia, là vaccine đầu tiên thử nghiệm lâm sàng giai đoạn 3 trên người.</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1255,12 +1255,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Gần 230 trẻ ở Bangladesh tử vong do bệnh sởi</t>
+          <t>Bé trai 4 tuổi nổi kín mụn nước toàn thân sau khi mắc cùng lúc zona thần kinh và thủy đậu</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Bangladesh đã ghi nhận 227 trường hợp tử vong ở trẻ em kể từ tháng 3, khi nước này đối mặt một trong những đợt bùng phát bệnh sởi tồi tệ nhất trong nhiều thập niên, theo AFP.</t>
+          <t>SKĐS - Bé trai 4 tuổi nhập viện trong tình trạng đau rát vùng lưng, bụng kèm các mụn nước mọc thành chùm rồi nhanh chóng lan khắp cơ thể. Đặc biệt, các bác sĩ xác định trẻ mắc đồng thời zona thần kinh và thủy đậu – tình trạng cực hiếm gặp ở trẻ khỏe mạnh.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1277,12 +1277,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Chuyên gia y tế tại Đà Nẵng cảnh báo về diễn tiến khó lường của sốt xuất huyết Dengue</t>
+          <t>Virus &amp;apos;bị lãng quên&amp;apos; ở người lớn quay trở lại tấn công từ mũi đến phổi</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Những ca sốt xuất huyết Dengue nặng tại Đà Nẵng trong thời gian qua cho thấy những diễn tiến khó lường của bệnh. Với những triệu chứng có thể chuyển biến nhanh, đòi hỏi cần phải được theo dõi sát sao và điều trị kịp thời.</t>
+          <t>Virus RSV không chỉ là mối đe dọa với trẻ nhỏ mà còn âm thầm gây biến chứng nặng, thậm chí tử vong ở người cao tuổi và bệnh nền nhưng bị xem nhẹ.</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1299,12 +1299,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Kiểm tra toàn bộ cơ sở tiêm vắc xin dịch vụ sau vụ tử vong do viêm não mô cầu</t>
+          <t>Nguy cơ cao nam giới bị nhiễm HIV do quan hệ tình dục đồng giới</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>TPO - Sở Y tế Cà Mau quyết định thành lập đoàn kiểm tra, giám sát công tác tiêm chủng tại các cơ sở dịch vụ trên toàn tỉnh, chấn chỉnh hoạt động quảng cáo trong tiêm chủng, sau khi tỉnh có 2 người mắc, trong đó 1 người tử vong do viêm não mô cầu.</t>
+          <t>Đó là một trong những thông tin từ Trung tâm Kiểm soát bệnh tật thành phố Huế nêu ra tại hội nghị triển khai chương trình phòng, chống HIV/AIDS năm 2026.</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1314,19 +1314,19 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Viêm não mô cầu: Từ sốt nhẹ đến tử vong chỉ trong vài giờ</t>
+          <t>Cảnh báo nhiều bệnh truyền nhiễm cùng lúc tăng mạnh ở TPHCM</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Viêm não mô cầu: Từ sốt nhẹ đến tử vong chỉ trong vài giờ</t>
+          <t>TPHCM đưa ra cảnh báo khi số ca sốt xuất huyết tăng hơn 70%, bệnh tay chân miệng tăng hơn 100% so với cùng kỳ năm ngoái. Đáng chú ý, cả hai bệnh truyền nhiễm đều ghi nhận ca tử vong.</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1336,19 +1336,19 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Nổi mẩn tưởng dị ứng thông thường, trẻ gặp nguy cơ tổn thương thận</t>
+          <t>Huế mở rộng xét nghiệm HIV, hướng tới chấm dứt dịch bệnh AIDS vào năm 2030</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>TPO - Nhiều trẻ phải nhập viện điều trị và ảnh hưởng đến cơ quan nội tạng chỉ từ những dấu hiệu ban đầu tưởng chừng đơn giản như ngứa và nổi mẩn đã gióng lên hồi chuông cảnh báo về sự chủ quan của không ít phụ huynh trước các biểu hiện bất thường của con trẻ.</t>
+          <t>SKĐS - Ngành Y tế TP Huế đang tiếp tục củng cố hệ thống phòng, chống HIV/AIDS, mở rộng xét nghiệm và nâng cao chất lượng điều trị nhằm hướng tới mục tiêu chấm dứt dịch bệnh AIDS vào năm 2030.</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1358,19 +1358,19 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Xuất hiện viêm não mô cầu, Đắk Lắk khẩn trương truy vết người tiếp xúc</t>
+          <t>Cập nhật ổ dịch vi rút Hanta</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Phát hiện ca tử vong do viêm não mô cầu, CDC Đắk Lắk đã phối hợp cùng cơ sở y tế địa phương tổ chức khử khuẩn, cấp thuốc kháng sinh dự phòng cho người tiếp xúc gần để ngăn chặn nguy cơ bùng phát dịch.</t>
+          <t>Tính đến ngày 14.5, tổng cộng đã có 11 người nghi nhiễm hoặc nhiễm vi rút Hanta liên quan du thuyền MV Hondius mang cờ Hà Lan, trong đó có 3 trường hợp tử vong, theo Tổ chức Y tế thế giới (WHO). Hiện chưa ghi nhận ca lây nhiễm nào bên ngoài du thuyền này.</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1387,12 +1387,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Viêm não mô cầu, 1 trẻ không qua khỏi</t>
+          <t>Bộ Y tế thông tin về chủng virus Hanta đang được WHO cảnh báo</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2 chú cháu trú tại phường Tân An, tỉnh Đắk Lắk dương tính với bệnh não mô cầu. Bệnh nặng khiến đứa trẻ không qua khỏi, còn người chú đang được cách ly điều trị.</t>
+          <t>SKĐS - Sau khi Tổ chức Y tế thế giới ghi nhận chùm ca nhiễm virus Hanta chủng Andes trên tàu du lịch quốc tế với 3 trường hợp tử vong, Bộ Y tế Việt Nam đã phát đi cảnh báo giám sát dịch tễ và khuyến cáo người dân không hoang mang nhưng cần chủ động phòng bệnh lây từ chuột sang người.</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1409,12 +1409,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Dịch bệnh tay chân miệng diễn biến phức tạp</t>
+          <t>TPHCM cảnh báo nguy cơ bùng phát nhiều bệnh truyền nhiễm mùa hè</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Cả nước ghi nhận hơn 34.000 ca mắc tính đến giữa tháng 4, trong đó có 8 trường hợp tử vong.</t>
+          <t>TPO - Hơn 16.000 ca sốt xuất huyết cùng số ca tay chân miệng tăng hơn gấp đôi so với cùng kỳ năm ngoái đang khiến TPHCM bước vào giai đoạn cảnh giác cao độ với dịch bệnh truyền nhiễm mùa hè.</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1431,12 +1431,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Cháu tử vong do não mô cầu, chú ruột 40 tuổi cũng nhiễm bệnh</t>
+          <t>Giám sát dịch bệnh ngay từ cửa khẩu và tại các cơ sở khám, chữa bệnh</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>TPO - Sau khi một cháu bé tử vong do viêm não mô cầu, ngành y tế Đắk Lắk lấy mẫu xét nghiệm, phát hiện thêm người chú ruột của cháu cũng dương tính.</t>
+          <t>Theo thông tin từ các cơ quan chức năng, tính đến chiều 14/5, Việt Nam chưa phát hiện trường hợp nào nhiễm virus Hanta.</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1446,19 +1446,19 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Phát hiện 2 bệnh nhân mắc viêm não mô cầu ở Đắk Lắk, 1 trường hợp tử vong</t>
+          <t>Việt Nam chưa phát hiện trường hợp nào nhiễm virus Hanta</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Ngày 27/4, Trung tâm Kiểm soát bệnh tật tỉnh Đắk Lắk cho biết, trên địa bàn tỉnh vừa ghi nhận 2 bệnh nhân mắc viêm não mô cầu , trong đó 1 trường hợp bệnh nhi đã tử vong.</t>
+          <t>(PLO)- Người phát ngôn Bộ Ngoại giao cho biết, theo thông tin từ các cơ quan chức năng, cho đến nay tại Việt Nam chưa phát hiện trường hợp nào nhiễm virus Hanta.</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1475,12 +1475,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Bé 2 tuổi tử vong do viêm não mô cầu, người thân phải cách ly y tế</t>
+          <t>TP.HCM cảnh báo bệnh sốt xuất huyết sẽ gia tăng</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Bé 2 tuổi tử vong do viêm não mô cầu, người thân phải cách ly y tế</t>
+          <t>(PLO)- Số ca tay chân miệng và sốt xuất huyết tăng, đã có trường hợp tử vong. Ngành y tế khuyến cáo người dân chủ động phòng bệnh, không chủ quan khi có triệu chứng nghi ngờ.</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1490,19 +1490,19 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Đắk Lắk: Bé trai 2 tuổi tử vong do mắc viêm não mô cầu</t>
+          <t>Hiếm gặp, bé trai 4 tuổi đồng thời mắc 2 bệnh do cùng 1 virus</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>(PLO)- Tỉnh Đắk Lắk vừa ghi nhận một trường hợp bệnh nhi tử vong do mắc viêm não mô cầu trong tình trạng thể tối cấp.</t>
+          <t>TPO - Bé trai 4 tuổi nhập viện trong tình trạng đau rát nhiều ở vùng lưng và bụng bên phải. Tại đây xuất hiện các cụm mụn nước, bọng nước tập trung trên nền da đỏ với kích thước khoảng 10x20 cm.</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1519,12 +1519,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Ghi nhận 2 ca mắc viêm não mô cầu, 1 trẻ tử vong</t>
+          <t>Khánh Hòa đã ghi nhận 2.254 ca tay chân miệng, bác sĩ khuyến cáo điều cần nhớ để phòng bệnh</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>(NLĐO) - Hai ca mắc viêm não mô cầu vừa được ghi nhận tại Đắk Lắk, trong đó 1 trẻ nhỏ đã tử vong, gióng lên cảnh báo về nguy cơ của bệnh truyền nhiễm nguy hiểm.</t>
+          <t>SKĐS - Thống kê từ đầu năm đến ngày 12/5, toàn tỉnh Khánh Hòa đã ghi nhận tổng cộng 2.254 ca tay chân miệng, trong đó có một số trường hợp nặng.</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1541,12 +1541,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Mỹ trấn an vi rút Hanta không phải COVID-19</t>
+          <t>Cúm dạ dày bùng phát trên du thuyền chở hơn 1.700 người</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Quyền giám đốc CDC của Mỹ trấn an vi rút Hanta không phải COVID-19, và những công dân trở về từ tàu du lịch có thể không cần thiết phải bị cách ly.</t>
+          <t>Cúm dạ dày bùng phát trên du thuyền Ambition chở hơn 1.700 người, và đã có một cụ ông lớn tuổi qua đời trên tàu này vì đau tim, theo Reuters ngày 13.5.</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1556,19 +1556,19 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Triệu chứng nhiễm virus Hanta dễ nhầm với các bệnh khác, làm gì để phòng ngừa?</t>
+          <t>Nguy cơ Ebola lây lan xuyên biên giới tại châu Phi</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Tổ chức Y tế Thế giới (WHO) virus Hanta là loại virus lây truyền từ động vật sang người, thường lây nhiễm tự nhiên ở loài gặm nhấm và đôi khi lây sang người. Thuộc họ Hantaviridae trong bộ Bunyavirales, mỗi chủng thường gắn với một loài vật chủ riêng, nơi chúng tồn tại nhưng gần như không gây biểu hiện rõ rệt.</t>
+          <t>Theo Bộ Y tế Uganda, bệnh nhân là một người đàn ông Congo 59 tuổi, nhập viện tại Bệnh viện Hồi giáo Kibuli ngày 11/5 và tử vong ngày 14/5. Nhà chức trách Uganda xác định, đây là ca bệnh nhập cảnh từ Cộng hòa Dân chủ (CHDC) Congo và cho biết, hiện chưa ghi nhận ca lây nhiễm trong cộng đồng tại Uganda.</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1578,19 +1578,19 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Sẽ xây dựng cơ chế đãi ngộ đặc thù cho lực lượng y tế tại hải đảo</t>
+          <t>Giám sát phòng tránh lây lan vi-rút Hanta</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>TPO - Chuyến công tác của Đoàn cán bộ Bộ Y tế tại Trường Sa (Khánh Hòa) còn là dịp ngành y tế khảo sát thực trạng hệ thống y tế cơ sở tại các điểm đảo thuộc đặc khu này.</t>
+          <t>Ngày 13/5, Cục Phòng bệnh (Bộ Y tế) cho biết: Theo Tổ chức Y tế Thế giới, tính đến ngày 8/5/2026, chùm ca bệnh do virus Hanta trên tàu MV Hondius đã ghi nhận tám trường hợp, trong đó ba người chết, đều được xác định là chủng vi-rút Andes (ANDV).</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1600,19 +1600,19 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Sốt cao mùa hè, cảnh giác viêm não Nhật Bản</t>
+          <t>Giảm nguy cơ lây bệnh lao trong cộng đồng</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Viêm não Nhật Bản thường tăng từ tháng 5 đến tháng 7, khởi đầu bằng sốt cao, đau đầu, nôn ói nên dễ bị nhầm với bệnh nhiễm trùng thông thường.</t>
+          <t>Tại Việt Nam, thách thức từ lao kháng thuốc và định kiến xã hội vẫn đang là rào cản ngăn người bệnh điều trị bệnh lao tại cộng đồng. Để có thể đạt mục tiêu cơ bản chấm dứt dịch bệnh lao vào năm 2030, ngành y tế cần tăng cường khám sàng lọc, phát hiện sớm bệnh lao, từ đó nâng cao hiệu quả điều trị, nhất là giảm nguy cơ lây lan trong cộng đồng.</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1629,12 +1629,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Khởi động điều tra tình trạng mù lòa, suy giảm thị lực trên toàn quốc</t>
+          <t>Pháp phong tỏa tàu chở hơn 1.700 người sau ca tử vong nghi do nhiễm virus</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>TPO - Tỉ lệ mù lòa và suy giảm thị lực tại Việt Nam đang đứng trước nhiều thay đổi do già hóa dân số và sự gia tăng của các bệnh không lây nhiễm. Trong bối cảnh đó, Bộ Y tế lần đầu triển khai lại cuộc điều tra quy mô toàn quốc về mù lòa sau hơn 10 năm, nhằm cập nhật thực trạng bệnh mắt trong cộng đồng và làm căn cứ xây dựng chính sách chăm sóc mắt giai đoạn mới.</t>
+          <t>Pháp phong tỏa tàu chở hơn 1.700 người sau ca tử vong nghi do nhiễm virus</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1644,19 +1644,19 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Bé gái vượt cửa tử khi men gan tăng gấp 100 lần</t>
+          <t>Bộ Y tế thông tin về chủng vi rút Hanta đang được WHO cảnh báo</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>TP HCM Rơi vào sốc sốt xuất huyết khiến men gan tăng vọt gấp 100 lần bình thường, bé gái 10 tuổi được bác sĩ Bệnh viện Nhi đồng 1 cứu sống ngoạn mục.</t>
+          <t>Trước các thông tin quốc tế liên quan đến chùm ca bệnh do vi rút Hanta ghi nhận trên tàu du lịch quốc tế MV Hondius, ngày 13-5, Cục Phòng bệnh Bộ Y tế có văn bản khẩn thông tin về tình hình dịch bệnh và khuyến cáo.</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1673,12 +1673,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Chuyên gia về hồi sức cảnh báo căn bệnh quen thuộc gây nguy kịch cho trẻ</t>
+          <t>Chùm ca nhiễm virus Hanta trên tàu du lịch: Bộ Y tế phát khuyến cáo khẩn</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>(NLĐO) - Một bé gái 10 tuổi bị sốc sốt xuất huyết Dengue nặng, men gan tăng gấp 100 lần bình thường vừa được các bác sĩ Bệnh viện Nhi Đồng 1 cứu sống thành công</t>
+          <t>(NLĐO) - Chùm ca nhiễm virus Hanta trên tàu MV Hondius khiến 3 người tử vong, Bộ Y tế khuyến cáo người dân theo dõi sức khỏe, chủ động phòng chống chuột.</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1695,12 +1695,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Virus Hanta: WHO khuyến nghị toàn bộ hành khách cách ly 42 ngày</t>
+          <t>Việt Nam chưa ghi nhận ca mắc virus Hanta</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Theo Thủ tướng Pháp Sebastien Lecornu, một trong năm hành khách người Pháp đã xuất hiện triệu chứng nhiễm virus Hanta trong chuyến bay hồi hương chiều 10/5. Ngoài ra, các chuyến bay đưa công dân Canada, Hà Lan, Thổ Nhĩ Kỳ, Anh, Ireland và Mỹ về nước cũng đang được thực hiện với các chuyến cuối cùng sẽ rời đi vào tối 11/5.</t>
+          <t>Chiều 13-5, Cục Phòng bệnh (Bộ Y tế) có công văn khẩn gửi các đơn vị chức năng của Bộ Y tế cập nhật thông tin về chùm ca bệnh do virus Hanta gây ra trên tàu du lịch quốc tế MV Hondius khi đang trên hành trình từ Argentina tới Cape Verde (quốc đảo ngoài khơi Tây Phi).</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -1710,19 +1710,19 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Thủy đậu biến chứng nhiễm khuẩn huyết, bé gái 6 tuổi nguy kịch</t>
+          <t>Khám sàng lọc lao cho người dân tại vùng cao</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>SKĐS - Khoa Nhi, Bệnh viện Bệnh Nhiệt đới Trung ương đang tích cực điều trị cho một bệnh nhi (6 tuổi, ở Lai Châu) nhập viện trong tình trạng suy hô hấp nặng và nhiễm khuẩn huyết do biến chứng thủy đậu.</t>
+          <t>Các bác sĩ Bệnh viện Phổi Trung ương vừa thực hiện gần 2.000 lượt khám sàng lọc lao cho người dân tại vùng cao, qua đó kịp thời phát hiện bệnh lao cũng như các bệnh lý khác để đưa vào điều trị, cũng như bảo vệ cộng đồng khỏi nguồn lây.</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1739,12 +1739,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Vaccine cúm mùa 2026 và sự biến đổi của virus cúm: Những thông tin cần biết</t>
+          <t>Hantavirus dễ nhầm với cúm có thể chuyển nặng nhanh</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Vaccine cúm mùa 2026 và sự biến đổi của virus cúm: Những thông tin cần biết</t>
+          <t>Một chùm ca nhiễm Hantavirus xuất hiện trên tàu du lịch quốc tế với 3 trường hợp tử vong đang khiến giới y tế toàn cầu lo ngại. Bệnh có biểu hiện ban đầu rất dễ nhầm với cúm.</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -1754,19 +1754,19 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Chung tay xây dựng hệ thống y tế bền vững</t>
+          <t>3 người tử vong trên tàu du lịch Hà Lan, Bộ Y tế khuyến cáo phòng bệnh từ chuột</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Châu Âu đang nỗ lực hỗ trợ châu Phi mở rộng năng lực sản xuất vắc-xin, qua đó góp phần bảo đảm an ninh y tế.</t>
+          <t>Trước thông tin về chùm ca bệnh do virus Hanta trên tàu du lịch Hà Lan, Cục Phòng bệnh (Bộ Y tế)  khuyến cáo người dân chủ động phòng bệnh, đặc biệt trong bối cảnh chuột phổ biến tại nhiều địa phương.</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -1776,19 +1776,19 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Tàu bùng phát vi rút Hanta sắp cập bến, WHO trấn an không phải 'COVID-19 thứ hai'</t>
+          <t>Phòng, chống virus Hanta: Việt Nam tăng cường giám sát tại cửa khẩu, cơ sở khám bệnh, chữa bệnh</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Tổng giám đốc Tổ chức Y tế thế giới (WHO) trực tiếp có mặt tại Tenerife (Tây Ban Nha) để giám sát chiến dịch sơ tán gần 150 hành khách từ tàu du lịch bùng phát vi rút Hanta, đồng thời trấn an người dân trên đảo này về nguy cơ lây nhiễm.</t>
+          <t>Bộ Y tế cho biết, hiện chưa ghi nhận công dân Việt Nam có liên quan đến chùm ca bệnh nhiễm virus Hanta. Cục Phòng bệnh đã có văn bản đề nghị các địa phương tăng cường giám sát tại cửa khẩu, giám sát tại cơ sở khám bệnh, chữa bệnh.</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -1798,19 +1798,19 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Không nên xem nhẹ thủy đậu, bác sĩ cảnh báo biến chứng nguy hiểm</t>
+          <t>3 người tử vong vì virus Hanta trên tàu du lịch, Việt Nam có nguy cơ?</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Nhiều phụ huynh vẫn xem thủy đậu là bệnh nhẹ, chủ yếu sợ để lại sẹo. Nhưng theo các chuyên gia truyền nhiễm, thực tế tại bệnh viện đang ghi nhận không ít trẻ biến chứng nặng như viêm phổi hoại tử, viêm não...</t>
+          <t>3 người tử vong vì virus Hanta trên tàu du lịch, Việt Nam có nguy cơ?</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1827,12 +1827,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Vắc xin có từ lâu, vì sao ca nhập viện do thủy đậu vẫn tăng?</t>
+          <t>Cách ly 42 ngày với người nguy cơ cao nhiễm virus Hanta</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Dù đã có vắc xin từ lâu, thủy đậu vẫn nằm trong nhóm bệnh truyền nhiễm phổ biến với hàng chục nghìn ca mỗi năm.</t>
+          <t>Với người tiếp xúc nguy cơ cao nhiễm virus Hanta, Tổ chức Y tế thế giới WHO khuyến cáo theo dõi chủ động và cách ly 42 ngày.</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -1849,12 +1849,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Lập quy hoạch chi tiết Trung tâm hành chính tỉnh Nghệ An</t>
+          <t>WHO cảnh báo chùm ca virus Hanta gây tử vong, Việt Nam tăng cường giám sát</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>TPO - Sở Xây dựng Nghệ An vừa đề xuất UBND tỉnh tiếp tục giao đơn vị tổ chức lập quy hoạch chi tiết tỷ lệ 1/500 Khu trung tâm hành chính tỉnh tại phường Vinh Lộc và xã Đông Lộc, tạo cơ sở triển khai dự án có tổng mức đầu tư gần 5.700 tỷ đồng.</t>
+          <t>Cục Phòng bệnh (Bộ Y tế) vừa phát công văn khẩn về bệnh do virus Hanta gây ra sau khi WHO ghi nhận chùm 11 ca bệnh trên tàu MV Hondius, trong đó có 3 ca tử vong.</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1864,19 +1864,19 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Cứu sống bệnh nhân trẻ mang 'quả mìn nổ chậm' trong não</t>
+          <t>Sốc sốt xuất huyết, bệnh nhi 10 tuổi suy đa cơ quan, tổn thương gan cấp tính nguy kịch</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>TPO - Đột ngột đau đầu dữ dội, nôn ói và mất thăng bằng, nam thanh niên 30 tuổi được đưa vào cấp cứu và phát hiện đồng thời khối dị dạng mạch máu não gây xuất huyết và hai túi phình động mạch não nguy hiểm.</t>
+          <t>SKĐS - Mới đây, Bệnh viện Nhi đồng 1 đã tiếp nhận và điều trị thành công cho một bé gái 10 tuổi mắc sốc sốt xuất huyết Dengue nặng, tổn thương gan cấp tính.</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1886,19 +1886,19 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Nguy cơ lây lan virus Ebola xuyên biên giới</t>
+          <t>Bệnh viện Hà Lan cách ly 12 nhân viên sau sự cố virus Hanta</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Theo phóng viên TTXVN tại châu Phi, ngày 15/5, Trung tâm Kiểm soát và phòng ngừa dịch bệnh châu Phi (ACDC) cho biết, Uganda đã phát hiện một ca nhiễm virus Ebola nhập cảnh từ Cộng hòa Dân chủ (CHDC) Congo, làm dấy lên lo ngại nguy cơ lây lan dịch bệnh xuyên biên giới.</t>
+          <t>Bệnh viện Hà Lan cách ly 12 nhân viên sau sự cố virus Hanta</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -1915,12 +1915,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Anime "Your Name." đưa những ký ức học trò đẹp nhất trở lại màn ảnh rộng</t>
+          <t>Biến chứng thủy đậu, bé trai 6 tuổi nhiễm khuẩn huyết, phải thở máy nguy kịch</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>HHTO - Từng tạo nên cơn sốt toàn cầu vào năm 2016, “Your Name.” chuẩn bị tái xuất màn ảnh rộng Việt Nam, đưa khán giả gặp lại Taki và Mitsuha trong câu chuyện hoán đổi thân xác đầy kỳ diệu.</t>
+          <t>SKĐS - Tin từ Bệnh viện Bệnh Nhiệt đới Trung ương, khoa Nhi của bệnh viện đang điều trị cho bệnh nhi 6 tuổi trong tình trạng rất nặng sau biến chứng thủy đậu.</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -1930,19 +1930,19 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Bộ Công Thương thúc tiến độ triển khai xăng E10</t>
+          <t>Vaccine cúm mùa 2026 và sự biến đổi của virus cúm: Những thông tin cần biết</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>TPO - Chỉ còn khoảng nửa tháng trước thời điểm bắt buộc bán xăng sinh học E10 trên phạm vi toàn quốc, Bộ Công Thương yêu cầu các doanh nghiệp đầu mối và phân phối xăng dầu khẩn trương chuẩn bị nguồn hàng, hệ thống phối trộn và cơ sở vật chất để sẵn sàng triển khai đồng loạt từ ngày 1/6.</t>
+          <t>Diễn biến phức tạp của virus cúm trong thời gian cuối năm 2025, đầu năm 2026 đang đặt ra yêu cầu cấp thiết về phòng bệnh chủ động. Các chuyên gia nhấn mạnh, tiêm vaccine cúm là giải pháp hiệu quả giúp giảm thiểu nguy cơ mắc bệnh cũng như các biến chứng nghiêm trọng.</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -1952,19 +1952,19 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Bệnh viện Phổi Bình Thuận nêu lý do xin miễn xử phạt sai sót đấu thầu thời điểm COVID-19</t>
+          <t>Manh mối dịch tễ về "bệnh nhân số 0" trong ổ dịch Hanta ở du thuyền hạng sang</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>(NLĐO) - Bệnh viện Phổi Bình Thuận giải trình vi phạm thủ tục đấu thầu vật tư chống dịch và đề nghị miễn xử phạt do xảy ra trong bối cảnh khẩn cấp</t>
+          <t>Theo New York Post, "bệnh nhân số 0" trong vụ bùng phát virus Hanta trên tàu du lịch đã được xác định là nhà điểu học người Hà Lan Leo Schilperoord (70 tuổi). Ông và vợ là bà Mirjam Schilperoord (69 tuổi) đều là những gương mặt quen thuộc trong cộng đồng nghiên cứu chim tại châu Âu.</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -1974,19 +1974,19 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Khởi tố ca sĩ Quang Lập và chủ Công ty BH Media</t>
+          <t>Một phụ nữ nhiễm bệnh nguy kịch, Pháp siết chặt kiểm soát virus Hanta</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Cục Cảnh sát điều tra tội phạm về tham nhũng, kinh tế, buôn lậu (C03, Bộ Công an) vừa ra quyết định khởi tố 5 vụ án hình sự liên quan đến hành vi xâm phạm quyền tác giả, quyền liên quan xảy ra tại nhiều công ty truyền thông, đơn vị giải trí.</t>
+          <t>Tổng thống Pháp Emmanuel Macron ngày 12/5 khẳng định tình hình liên quan đến virus Hanta tại Pháp vẫn “nằm trong tầm kiểm soát” của chính phủ, trong bối cảnh một phụ nữ Pháp nhiễm bệnh đang trong tình trạng nguy kịch và nhiều nước châu Âu tăng cường các biện pháp phòng dịch.</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -1996,19 +1996,19 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Mỹ tuyên bố tiêu diệt phó chỉ huy toàn cầu của ISIS trong chiến dịch tại Nigeria</t>
+          <t>Hà Lan cách ly 12 nhân viên y tế sau sự cố xử lý ca nhiễm virus Hanta</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Trong bài đăng trên mạng xã hội Truht social tối 15/5, Tổng thống Mỹ cho biết chiến dịch được thực hiện theo chỉ thị trực tiếp của ông và ca ngợi đây là “một nhiệm vụ được lên kế hoạch tỉ mỉ và rất phức tạp”.</t>
+          <t>Vụ việc xảy ra tại bệnh viện Radboudumc ở thành phố Nijmegen, nơi tiếp nhận một hành khách từ tàu du lịch MV Hondius vào ngày 7/5. Theo thông báo của bệnh viện, máu và nước tiểu của bệnh nhân đã được xử lý mà không thực hiện đầy đủ các quy trình an toàn nghiêm ngặt, dẫn đến việc 12 nhân viên y tế phải cách ly phòng ngừa trong thời gian 6 tuần.</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -2018,19 +2018,19 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>VNVC tặng kho bảo quản vaccine chuẩn quốc tế cho đặc khu Côn Đảo</t>
+          <t>Thái Lan siết chặt kiểm tra y tế tại sân bay quốc tế để ngăn chặn virus Hanta</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Sáng 16-5, Hệ thống Trung tâm Tiêm chủng VNVC đã trao tặng đặc khu Côn Đảo (TPHCM) gói tài trợ hơn 10 tỷ đồng, gồm: tiêm miễn phí vaccine cúm cho toàn bộ quân và dân đảo trong 3 năm liên tiếp, tặng 1 kho lạnh bảo quản vaccine đạt chuẩn quốc tế và cam kết ưu tiên cung ứng đầy đủ các vaccine thế hệ mới.</t>
+          <t>Cục trưởng DDC, Tiến sĩ Montien Kanasawadse, cho biết quyết định tăng cường quy trình sàng lọc sức khỏe đối với hành khách nhập cảnh từ các quốc gia và vùng lãnh thổ Nam Mỹ tại các sân bay quốc tế lớn, vừa để trấn an công chúng, vừa khẳng định chính phủ đã triển khai đầy đủ các bước phòng ngừa cần thiết, dù đến nay chưa ghi nhận ca nhiễm virus Hanta nào tại Thái Lan. Ông Montien nhấn mạnh, động thái này cũng nhằm bảo đảm môi trường du lịch an toàn.</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2040,19 +2040,19 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Tăng cường năng lực y tế dự phòng cho Đặc khu Côn Đảo</t>
+          <t>Bé trai 6 tuổi nguy kịch vì biến chứng nặng từ thủy đậu</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Trong định hướng phát triển Đặc khu Côn Đảo, nâng cao năng lực y tế dự phòng được xác định là nhiệm vụ quan trọng nhằm bảo vệ sức khỏe cộng đồng và phát triển bền vững vùng biển đảo. Chương trình hỗ trợ vaccine và hạ tầng bảo quản hiện đại là bước đi cụ thể cho định hướng chuyển từ chữa bệnh sang chủ động phòng bệnh.</t>
+          <t>TPO - Từ những nốt phỏng nước tưởng chừng thông thường do thủy đậu, một bé trai 6 tuổi ở Lai Châu đã rơi vào tình trạng nguy kịch với suy hô hấp nặng, nhiễm khuẩn huyết do phế cầu và phải thở máy xâm nhập.</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2062,19 +2062,19 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>unsure</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Viêm gan B có gây rụng tóc?</t>
+          <t>WHO tuyên bố 'tình trạng khẩn cấp sức khỏe cộng đồng gây lo ngại quốc tế' liên quan dịch Ebola</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Tôi bị viêm gan B mạn tính, đang điều trị và theo dõi. Gần đây, tóc tôi rụng nhiều có phải do viêm gan B không? (Thanh Mai, Tây Ninh)</t>
+          <t>(PLO)- Tổ chức Y tế Thế giới (WHO) tuyên bố dịch Ebola bùng phát tại Cộng hòa Dân chủ Congo và Uganda là "tình trạng khẩn cấp về sức khỏe cộng đồng gây lo ngại quốc tế", sau khi ghi nhận lượng lớn trường hợp nghi nhiễm và tử vong ở hai nước này.</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2084,19 +2084,19 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Virus Hanta lây qua phân, nước tiểu chuột: Chuyên gia khuyến cáo người dân</t>
+          <t>Bé gái bị cô đặc máu vì bệnh truyền nhiễm, cảnh báo biến chứng chết người</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Phó Giáo sư, Tiến sĩ Trần Đắc Phu cho biết, virus Hanta có thể gây hội chứng sốt xuất huyết kèm suy thận hoặc suy tim phổi nguy hiểm. Dù Việt Nam chưa ghi nhận ổ dịch điển hình, ngành y tế vẫn tăng cường giám sát nguy cơ xâm nhập.</t>
+          <t>TPO - Liên tục tiếp nhận trẻ bị sốc sốt xuất huyết Dengue nặng, Bệnh viện Nhi Đồng 1 cảnh báo nhiều ca có thể diễn tiến thành suy đa cơ quan, tử vong rất nhanh. Đáng lo ngại, số ca mắc tại TPHCM hiện đã tăng hơn 70% so với cùng kỳ năm ngoái.</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2113,12 +2113,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Thời tiết diễn biến phức tạp, Hà Tĩnh chủ động ngăn dịch sốt xuất huyết</t>
+          <t>Số ca mắc viêm phổi do virus gia tăng</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>SKĐS - Thời tiết diễn biến thất thường, Hà Tĩnh đang ghi nhận hai ổ dịch sốt xuất huyết. Ngành y tế địa phương đang triển khai nhiều giải pháp nhằm khoanh vùng, xử lý ổ dịch, hạn chế nguy cơ lây lan diện rộng.</t>
+          <t>Trung tâm Kiểm soát bệnh tật TPHCM (HCDC) vừa có văn bản gửi các bệnh viện công lập và ngoài công lập trên địa bàn nhằm tăng cường giám sát viêm phổi nặng do virus (SVP) trên địa bàn thành phố.</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2135,12 +2135,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Hà Tĩnh tăng cường giám sát, phòng chống bệnh do virus Hanta</t>
+          <t>Cập nhật vi rút hanta trên du thuyền: Canada ghi nhận ca nghi nhiễm</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>SKĐS - Trước nguy cơ bệnh do virus Hanta xâm nhập và lây lan, ngành y tế Hà Tĩnh tăng cường giám sát, chủ động triển khai các biện pháp phòng chống.</t>
+          <t>Các quan chức y tế Canada cho biết một trong 4 công dân nước này đang cách ly tại tỉnh British Columbia sau khi tiếp xúc với vi rút hanta trên du thuyền MV Hondius đã có kết quả dương tính.</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2157,12 +2157,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CEO Nvidia gây sốt mạng xã hội với khoảnh khắc ăn mì trên đường phố Bắc Kinh</t>
+          <t>Người dân Côn Đảo được tiêm ngừa cúm miễn phí ba năm</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>CEO Nvidia Jensen Huang gây chú ý khi xuất hiện bất ngờ tại một ngõ nhỏ Bắc Kinh, thoải mái thưởng thức mì và ẩm thực đường phố như một du khách bình thường.</t>
+          <t>VNVC tài trợ hơn 10 tỷ đồng cho Côn Đảo, tiêm miễn phí vaccine cúm trong ba năm và đầu tư kho lạnh bảo quản vaccine đạt chuẩn GSP đầu tiên.</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2172,19 +2172,19 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>unsure</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Vaccine sốt rét không cần bảo quản lạnh</t>
+          <t>Thái Lan xếp vi rút Hanta vào nhóm bệnh nguy hiểm, cách ly người tiếp xúc 42 ngày</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Các nhà nghiên cứu từ Đại học Griffith (Australia) vừa phát triển thành công vaccine sốt rét thế hệ mới không yêu cầu bảo quản lạnh. Đây là bước tiến quan trọng vì bệnh sốt rét hiện cướp đi sinh mạng của hơn 500.000 người mỗi năm trên thế giới, chủ yếu tại những quốc gia đang phát triển.</t>
+          <t>Thái Lan xếp vi rút Hanta vào nhóm bệnh nguy hiểm, yêu cầu báo ca nghi nhiễm trong 3 giờ và cách ly người tiếp xúc 42 ngày.</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2194,19 +2194,19 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Điều tra: Thịt bẩn luồn lách đến bữa ăn - Kỳ 3: Thịt heo chết vào lò lạp xưởng</t>
+          <t>VNVC tài trợ kho lạnh và 3 năm tiêm cúm cho Côn Đảo</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>(PLO)- Từ những bãi đất trống ven đường, hàng trăm ký thịt heo không rõ nguồn gốc được mua bán, giao dịch ngay giữa đường trong đêm khuya.</t>
+          <t>Sáng 16-5, Hệ thống Trung tâm Tiêm chủng VNVC đã trao tặng Đặc khu Côn Đảo Gói tài trợ đặc biệt về tiêm chủng vắc xin, trị giá hơn 10 tỉ đồng, góp phần bảo vệ sức khỏe toàn quân, dân Côn Đảo.</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2216,19 +2216,19 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Bệnh viện Phổi Bình Thuận giải trình về vi phạm đấu thầu trong phòng chống dịch</t>
+          <t>Cẩn trọng với sốt xuất huyết Dengue: Thực tế từ những ca bệnh nặng tại Hải Phòng</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>TPO - Liên quan việc bị xác định có vi phạm hành chính trong lĩnh vực kế hoạch và đầu tư về đấu thầu, Bệnh viện Phổi Bình Thuận đã có văn bản gửi Sở Tài chính tỉnh Lâm Đồng để giải trình nguyên nhân dẫn đến sai sót trong quá trình mua sắm phục vụ phòng, chống dịch COVID-19.</t>
+          <t>Cẩn trọng với sốt xuất huyết Dengue: Thực tế từ những ca bệnh nặng tại Hải Phòng</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2238,19 +2238,19 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Hà Nội: "Đi từng ngõ, gõ từng nhà" chặn dịch sắp vào cao điểm</t>
+          <t>Khởi động 'Ký ức COVID-19', sẵn sàng ứng phó dịch bệnh trong tương lai</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>(Dân trí) - Những năm gần đây, số ca mắc sốt xuất huyết có xu hướng gia tăng, với các ổ dịch không chỉ tập trung tại nội thành mà còn lan rộng ra ngoại thành.</t>
+          <t>(PLO)- TP.HCM khởi động chương trình Ký ức COVID-19, xây dựng kho dữ liệu, nâng cao năng lực sẵn sàng ứng phó dịch bệnh trong tương lai.</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2260,19 +2260,19 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>unsure</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Bệnh viện Phổi Bình Thuận đề nghị miễn xử phạt do vi phạm thủ tục đấu thầu</t>
+          <t>Cẩn trọng với sốt xuất huyết Dengue: Thực tế từ những ca bệnh nặng tại Hải Phòng</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Ngày 15-5, Bệnh viện Phổi Bình Thuận cho biết đã có văn bản gửi Sở Tài chính tỉnh Lâm Đồng giải trình các sai sót trong đấu thầu mua sắm vật tư phòng, chống dịch Covid-19 giai đoạn 2020-2021; đồng thời đề nghị xem xét miễn xử phạt vi phạm hành chính do vụ việc xảy ra trong “tình thế cấp thiết” thời điểm dịch bệnh.</t>
+          <t>Những câu chuyện thực tế tại Hải Phòng cho thấy sốt xuất huyết Dengue hiện không còn là bệnh xâm nhập, mà đã trở thành bệnh lưu hành, hiện hữu quanh năm tại địa phương. Việc thiếu các biện pháp phòng ngừa chủ động hoặc chậm trễ trong quá trình điều trị có thể khiến bệnh chuyển biến nặng và nguy cơ dẫn đến tử vong.</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2282,19 +2282,19 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Vaccine cúm gia cầm đầu tiên thử nghiệm trên người giai đoạn 3</t>
+          <t>Cúm B tấn công người già, bệnh nền: Nhiều bệnh nhân nhập viện trong tình trạng nặng</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Thử nghiệm được tổ chức tại Anh và Mỹ, dự kiến có 4.000 người tham gia, là vaccine đầu tiên thử nghiệm lâm sàng giai đoạn 3 trên người.</t>
+          <t>Các ca bệnh cúm B nằm điều trị tại Bệnh viện Bệnh Nhiệt đới Trung ương hầu hết đều rơi vào tình trạng biến chứng nặng do có bệnh lý nền, người cao tuổi với điểm chung là triệu chứng ban đầu âm thầm nhưng nhanh chóng tiến triển suy hô hấp.</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2311,12 +2311,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Bé trai 4 tuổi nổi kín mụn nước toàn thân sau khi mắc cùng lúc zona thần kinh và thủy đậu</t>
+          <t>Sốt xuất huyết Dengue tại Hải Phòng: Cẩn trọng với diễn biến khó lường của bệnh</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>SKĐS - Bé trai 4 tuổi nhập viện trong tình trạng đau rát vùng lưng, bụng kèm các mụn nước mọc thành chùm rồi nhanh chóng lan khắp cơ thể. Đặc biệt, các bác sĩ xác định trẻ mắc đồng thời zona thần kinh và thủy đậu – tình trạng cực hiếm gặp ở trẻ khỏe mạnh.</t>
+          <t>Diễn biến sốt xuất huyết Dengue tại Hải Phòng những năm gần đây cho thấy rõ sự khó lường của dịch bệnh. Theo các chuyên gia, ngay cả thời điểm dịch yên ắng cũng ẩn chứa rất nhiều nguy cơ, người dân tuyệt đối không chủ quan.</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -2333,12 +2333,12 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Lan truyền nguy hiểm dùng nước tiểu chữa bệnh, bác sĩ sửng sốt, cảnh báo nóng</t>
+          <t>Cảnh báo nhiều ca cúm B suy hô hấp: Bác sĩ chỉ điểm chung nguy hiểm</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Những chia sẻ nguy hiểm về việc dùng nước tiểu để tắm, rửa mặt hay thậm chí nhỏ mắt đang gây xôn xao mạng xã hội, nhưng lại được một số người ca ngợi như “bài thuốc tự nhiên” chữa bệnh.</t>
+          <t>Cảnh báo nhiều ca cúm B suy hô hấp: Bác sĩ chỉ điểm chung nguy hiểm</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2348,19 +2348,19 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Virus &amp;apos;bị lãng quên&amp;apos; ở người lớn quay trở lại tấn công từ mũi đến phổi</t>
+          <t>Một đợt khám sức khỏe cộng đồng, phát hiện 171 ca nghi mắc lao</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Virus RSV không chỉ là mối đe dọa với trẻ nhỏ mà còn âm thầm gây biến chứng nặng, thậm chí tử vong ở người cao tuổi và bệnh nền nhưng bị xem nhẹ.</t>
+          <t>Một đợt khám sức khỏe cộng đồng, phát hiện 171 ca nghi mắc lao</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2377,12 +2377,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Tiết canh vịt khiến 31 người ngộ độc</t>
+          <t>Vì sao bệnh tay chân miệng tăng mạnh ở trẻ mầm non vào đầu tuần?</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Hưng Yên 31 người nhập viện với dấu hiệu nôn mửa, đau bụng, tiêu chảy, sốt sau khi ăn món tiết canh vịt tại xã Quỳnh Phụ.</t>
+          <t>SKĐS - Bệnh tay chân miệng đang có xu hướng gia tăng ở trẻ mầm non. Nhận biết sớm dấu hiệu giúp cha mẹ xử lý kịp thời, tránh biến chứng nguy hiểm.</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2392,19 +2392,19 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Cặp cá voi kiếm ăn ở biển Đăk Lăk</t>
+          <t>Bệnh tay chân miệng xuất hiện ở 126 xã, phường, Hà Nội kích hoạt chiến dịch phòng dịch trong trường học</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Hai con cá voi dài khoảng 7-10 m xuất hiện kiếm ăn gần đảo Cù Lao Mái Nhà, xã Ô Loan, thu hút người dân và du khách theo dõi, sáng 15/5.</t>
+          <t>SKĐS - Trước nguy cơ bệnh tay chân miệng gia tăng, đặc biệt ở trẻ dưới 5 tuổi, Hà Nội phát động chiến dịch vệ sinh, khử khuẩn tại các trường mầm non nhằm giảm thiểu lây nhiễm và bảo vệ sức khỏe trẻ em.</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -2414,19 +2414,19 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Nguy cơ cao nam giới bị nhiễm HIV do quan hệ tình dục đồng giới</t>
+          <t>Ổ dịch não mô cầu làm một người tử vong ở Cà Mau đã được dập</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Đó là một trong những thông tin từ Trung tâm Kiểm soát bệnh tật thành phố Huế nêu ra tại hội nghị triển khai chương trình phòng, chống HIV/AIDS năm 2026.</t>
+          <t>Ngày 20-4, Trung tâm Kiểm soát bệnh tật tỉnh Cà Mau cho biết đã kết thúc ổ dịch do bệnh não mô cầu liên quan Trại giam Cái Tàu, xã Khánh An, tỉnh Cà Mau. Ổ dịch này đã làm một người tử vong.</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -2443,12 +2443,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Cảnh báo nhiều bệnh truyền nhiễm cùng lúc tăng mạnh ở TPHCM</t>
+          <t>6 bệnh truyền nhiễm nguy hiểm cần phòng ngừa sớm ở trẻ dưới 1 tuổi</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>TPHCM đưa ra cảnh báo khi số ca sốt xuất huyết tăng hơn 70%, bệnh tay chân miệng tăng hơn 100% so với cùng kỳ năm ngoái. Đáng chú ý, cả hai bệnh truyền nhiễm đều ghi nhận ca tử vong.</t>
+          <t>Hệ miễn dịch của trẻ dưới 1 tuổi non yếu, trong khi 6 bệnh truyền nhiễm nguy hiểm như bạch hầu, ho gà, uốn ván, bại liệt, viêm gan B và Hib chực chờ tấn công.</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2465,12 +2465,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Ngoại trưởng Mỹ gây sốt với khoảnh khắc 'ngỡ ngàng' trong Đại lễ đường Nhân dân</t>
+          <t>Khống chế ổ dịch viêm não mô cầu tại trại giam ở Cà Mau</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Ngoại trưởng Mỹ gây chú ý với khoảnh khắc tỏ ra ngỡ ngàng và nhiều lần chỉ tay lên trần nhà trong Đại lễ đường Nhân dân ở Bắc Kinh.</t>
+          <t>Trung tâm Kiểm soát bệnh tật (CDC) tỉnh Cà Mau thông báo đã khống chế ổ dịch viêm não mô cầu tại Trại giam Cái Tàu, xã Khánh An, sau thời gian giám sát và xử lý.</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2480,19 +2480,19 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Huế mở rộng xét nghiệm HIV, hướng tới chấm dứt dịch bệnh AIDS vào năm 2030</t>
+          <t>Ổ dịch não mô cầu ở Cà Mau đã được kiểm soát</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>SKĐS - Ngành Y tế TP Huế đang tiếp tục củng cố hệ thống phòng, chống HIV/AIDS, mở rộng xét nghiệm và nâng cao chất lượng điều trị nhằm hướng tới mục tiêu chấm dứt dịch bệnh AIDS vào năm 2030.</t>
+          <t>Ngày 20/4, đại diện CDC Mau thông tin, ổ dịch đã được kiểm soát sau 10 ngày kể từ phát hiện ca bệnh, không ghi nhận thêm trường hợp mắc mới liên quan đến ổ dịch.</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2509,12 +2509,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Điều tra: Thịt bẩn luồn lách đến bữa ăn - Kỳ 2: Đường đi của xe chở thịt heo chết lúc rạng sáng</t>
+          <t>Khống chế thành công ổ dịch viêm não mô cầu ở Cà Mau</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>(PLO)- Từ lò mổ chui, những túi thịt heo chết được chia nhỏ, vận chuyển bằng xe máy hoặc xe tải len lỏi vào một số cơ sở cung cấp suất ăn công nghiệp.</t>
+          <t>TPO - Trung tâm Kiểm soát bệnh tật tỉnh Cà Mau xác nhận, ổ dịch viêm não mô cầu tại Trại giam Cái Tàu đã được kiểm soát, kết thúc thời gian giám sát và cách ly.</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -2524,19 +2524,19 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Cập nhật ổ dịch vi rút Hanta</t>
+          <t>Cà Mau cập nhật thông tin vụ 2 ca não mô cầu</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Tính đến ngày 14.5, tổng cộng đã có 11 người nghi nhiễm hoặc nhiễm vi rút Hanta liên quan du thuyền MV Hondius mang cờ Hà Lan, trong đó có 3 trường hợp tử vong, theo Tổ chức Y tế thế giới (WHO). Hiện chưa ghi nhận ca lây nhiễm nào bên ngoài du thuyền này.</t>
+          <t>(NLĐO) – CDC tỉnh Cà Mau đã có thông báo liên quan đến 2 ca dương tính với não mô cầu tại Trại giam Cái Tàu.</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2553,12 +2553,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Bộ Y tế thông tin về chủng virus Hanta đang được WHO cảnh báo</t>
+          <t>Cà Mau công bố kết thúc ổ dịch não mô cầu liên quan trại giam Cái Tàu</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>SKĐS - Sau khi Tổ chức Y tế thế giới ghi nhận chùm ca nhiễm virus Hanta chủng Andes trên tàu du lịch quốc tế với 3 trường hợp tử vong, Bộ Y tế Việt Nam đã phát đi cảnh báo giám sát dịch tễ và khuyến cáo người dân không hoang mang nhưng cần chủ động phòng bệnh lây từ chuột sang người.</t>
+          <t>(PLO)- Đến ngày 20-4, ổ dịch não mô cầu liên quan trại giam Cái Tàu không phát sinh ca mắc mới, được xác định đủ điều kiện kết thúc theo quy định.</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -2575,12 +2575,12 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>TPHCM cảnh báo nguy cơ bùng phát nhiều bệnh truyền nhiễm mùa hè</t>
+          <t>Sốt xuất huyết Dengue tại miền Trung - Tây Nguyên: Không chỉ mùa mưa, không chừa độ tuổi</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>TPO - Hơn 16.000 ca sốt xuất huyết cùng số ca tay chân miệng tăng hơn gấp đôi so với cùng kỳ năm ngoái đang khiến TPHCM bước vào giai đoạn cảnh giác cao độ với dịch bệnh truyền nhiễm mùa hè.</t>
+          <t>Sốt xuất huyết Dengue tại miền Trung - Tây Nguyên: Không chỉ mùa mưa, không chừa độ tuổi</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -2597,12 +2597,12 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Giám sát dịch bệnh ngay từ cửa khẩu và tại các cơ sở khám, chữa bệnh</t>
+          <t>Nguy cơ rối loạn điện giải, viêm phổi mùa nắng nóng</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Theo thông tin từ các cơ quan chức năng, tính đến chiều 14/5, Việt Nam chưa phát hiện trường hợp nào nhiễm virus Hanta.</t>
+          <t>(PLO)- Từ đầu tháng 4, miền Nam bước vào giai đoạn nắng nóng diện rộng với nền nhiệt phổ biến 35–37°C.</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -2619,12 +2619,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Việt Nam chưa phát hiện trường hợp nào nhiễm virus Hanta</t>
+          <t>Bệnh "sốt đất" khiến hàng chục người ở Thái Lan tử vong nguy hiểm ra sao?</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>(PLO)- Người phát ngôn Bộ Ngoại giao cho biết, theo thông tin từ các cơ quan chức năng, cho đến nay tại Việt Nam chưa phát hiện trường hợp nào nhiễm virus Hanta.</t>
+          <t>Bệnh "sốt đất" khiến hàng chục người ở Thái Lan tử vong nguy hiểm ra sao?</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -2634,19 +2634,19 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>relevant</t>
+          <t>unsure</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>TP.HCM cảnh báo bệnh sốt xuất huyết sẽ gia tăng</t>
+          <t>Đau xót: Bé gái 11 tuổi tử vong do viêm màng não mô cầu thể tối cấp</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>(PLO)- Số ca tay chân miệng và sốt xuất huyết tăng, đã có trường hợp tử vong. Ngành y tế khuyến cáo người dân chủ động phòng bệnh, không chủ quan khi có triệu chứng nghi ngờ.</t>
+          <t>SKĐS - Theo báo cáo của Trung tâm Kiểm soát Bệnh tật TP.HCM (HCDC), qua điều tra dịch tễ tuần 14 (30/3-5/4), thành phố ghi nhận một trường hợp tại phường Hòa Hưng là bé gái 11 tuổi mắc viêm màng não mô cầu không qua khỏi.</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -2663,12 +2663,12 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Nhiều người bị suy giảm thị lực hoặc mù mắt do chơi Pickleball</t>
+          <t>Sàng lọc cộng đồng tại Nghệ An phát hiện 171 ca nghi mắc bệnh lao</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>TPO - Sau cú va chạm với bóng khi chơi Pickleball, một người đàn ông 39 tuổi phải nhập viện trong tình trạng xuất huyết mắt, thị lực suy giảm nghiêm trọng, trong khi một trường hợp khác đã mất vĩnh viễn một bên mắt do vỡ nhãn cầu. Các bác sĩ cảnh báo chấn thương mắt liên quan đến Pickleball đang gia tăng và có thể để lại hậu quả nặng nề nếu người chơi chủ quan.</t>
+          <t>SKĐS - Việc đưa hoạt động khám sàng lọc xuống tận cộng đồng đang chứng minh hiệu quả rõ nét trong phòng, chống bệnh lao. Chỉ trong một tuần tại Nghĩa Đàn (Nghệ An), Bệnh viện Phổi Nghệ An đã phát hiện 171 trường hợp nghi mắc – những ca bệnh có nguy cơ bị bỏ sót nếu người dân không được tiếp cận kịp thời dịch vụ y tế.</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -2678,19 +2678,19 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Tỷ phú Elon Musk gây sốt với màn check-in ngẫu hứng trước Đại lễ đường Nhân dân</t>
+          <t>Gần một nửa ca viêm não mô cầu dưới 15 tuổi, cảnh báo nguy cơ cao</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Video lan truyền trên mạng cho thấy ông Musk đứng cùng nhiều lãnh đạo doanh nghiệp và quan chức Mỹ, trong đó có Bộ trưởng Quốc phòng Pete Hegseth và Giám đốc điều hành Apple Tim Cook. Trong lúc mọi người xếp hàng chụp ảnh lưu niệm trước Đại lễ đường Nhân dân, ông Musk bất ngờ giơ điện thoại lên, xoay chậm một vòng để ghi lại khung cảnh xung quanh.</t>
+          <t>Theo thống kê từ Bộ Y tế, đầu năm đến nay cả nước ghi nhận 24 ca mắc bệnh viêm não mô cầu, đáng lưu ý, trẻ dưới 15 tuổi chiếm tới 46% tổng số ca mắc.</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -2700,19 +2700,19 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Hiếm gặp, bé trai 4 tuổi đồng thời mắc 2 bệnh do cùng 1 virus</t>
+          <t>TP.HCM: Bé hơn 2 tuổi tử vong do viêm màng não mô cầu thể tối cấp, diễn tiến rất nhanh</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>TPO - Bé trai 4 tuổi nhập viện trong tình trạng đau rát nhiều ở vùng lưng và bụng bên phải. Tại đây xuất hiện các cụm mụn nước, bọng nước tập trung trên nền da đỏ với kích thước khoảng 10x20 cm.</t>
+          <t>Em bé hơn 2 tuổi ở TP.HCM mắc viêm màng não mô cầu thể tối cấp, bệnh diễn tiến nhanh, dù được điều trị nhưng không qua khỏi.</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -2729,12 +2729,12 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Điều gì khiến Hantavirus trở thành mối lo y tế dù ít gặp?</t>
+          <t>Ghi nhận 1 ca tử vong do não mô cầu tại TP.HCM</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>SKĐS - Virus Hanta là tác nhân có thể gây tổn thương phổi hoặc suy thận nghiêm trọng ở người, với tỷ lệ tử vong cao ở một số trường hợp nặng. Dù bệnh tương đối hiếm gặp, các chuyên gia vẫn cảnh báo cần chú ý nguy cơ lây nhiễm từ động vật gặm nhấm và môi trường sống xung quanh...</t>
+          <t>(PLO)- TP.HCM ghi nhận một ca bệnh nhi hơn 2 tuổi tử vong sau khởi phát bệnh não mô cầu không lâu dù đã được điều trị tích cực.</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -2744,19 +2744,19 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Khánh Hòa đã ghi nhận 2.254 ca tay chân miệng, bác sĩ khuyến cáo điều cần nhớ để phòng bệnh</t>
+          <t>TP.HCM: Hơn 1.300 ca tay chân miệng trong một tuần, cao hơn ngưỡng cảnh báo</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>SKĐS - Thống kê từ đầu năm đến ngày 12/5, toàn tỉnh Khánh Hòa đã ghi nhận tổng cộng 2.254 ca tay chân miệng, trong đó có một số trường hợp nặng.</t>
+          <t>Trong một tuần, TP.HCM ghi nhận 1.347 ca bệnh tay chân miệng, tăng 64% so với trung bình 4 tuần trước (821 ca). Có 43/168 phường, xã, đặc khu có số ca mắc tăng báo động.</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -2773,12 +2773,12 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Cúm dạ dày bùng phát trên du thuyền chở hơn 1.700 người</t>
+          <t>Bệnh sởi ở người lớn: Triệu chứng, biến chứng và cách phòng ngừa</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Cúm dạ dày bùng phát trên du thuyền Ambition chở hơn 1.700 người, và đã có một cụ ông lớn tuổi qua đời trên tàu này vì đau tim, theo Reuters ngày 13.5.</t>
+          <t>Người nhà chị N.T.B cho biết, khoảng 10 ngày trước khi khởi phát bệnh, cháu gái sống cùng chị N.T.B mắc sởi và đã điều trị khỏi. Tuy nhiên, chị B không thực hiện các biện pháp phòng ngừa. Cách thời điểm nhập viện 4 ngày, chị bắt đầu sốt cao 38,5–39°C nhưng tự mua thuốc hạ sốt điều trị tại nhà.</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -2795,12 +2795,12 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Nguy cơ Ebola lây lan xuyên biên giới tại châu Phi</t>
+          <t>Bệnh tay chân miệng: Số ca bệnh nặng có thể tiếp tục gia tăng</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Theo Bộ Y tế Uganda, bệnh nhân là một người đàn ông Congo 59 tuổi, nhập viện tại Bệnh viện Hồi giáo Kibuli ngày 11/5 và tử vong ngày 14/5. Nhà chức trách Uganda xác định, đây là ca bệnh nhập cảnh từ Cộng hòa Dân chủ (CHDC) Congo và cho biết, hiện chưa ghi nhận ca lây nhiễm trong cộng đồng tại Uganda.</t>
+          <t>Ông Võ Hải Sơn, Phó Cục trưởng Cục Phòng bệnh, Bộ Y tế đã trả lời báo chí về dịch bệnh tay chân miệng.</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -2817,12 +2817,12 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Từ cơn sốt nhẹ đến giây phút sinh tử - 24 giờ mong manh của con trước bệnh do não mô cầu</t>
+          <t>"Bệnh trẻ em" khiến người phụ nữ toàn thân chuyển đỏ, biến chứng hô hấp</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Bệnh do não mô cầu đe dọa tính mạng trẻ nếu không được phát hiện và điều trị kịp thời. Đáng lo ngại hơn, 4 nhóm huyết thanh A, C, Y, W gây bệnh đang lưu hành tại Việt Nam.</t>
+          <t>"Bệnh trẻ em" khiến người phụ nữ toàn thân chuyển đỏ, biến chứng hô hấp</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -2832,19 +2832,19 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Giám sát phòng tránh lây lan vi-rút Hanta</t>
+          <t>Người lớn gặp biến chứng nặng vì chủ quan bệnh sởi chỉ gặp ở trẻ em</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Ngày 13/5, Cục Phòng bệnh (Bộ Y tế) cho biết: Theo Tổ chức Y tế Thế giới, tính đến ngày 8/5/2026, chùm ca bệnh do virus Hanta trên tàu MV Hondius đã ghi nhận tám trường hợp, trong đó ba người chết, đều được xác định là chủng vi-rút Andes (ANDV).</t>
+          <t>Theo người nhà, khoảng 10 ngày trước khi khởi phát bệnh, cháu gái sống cùng nhà mắc sởi và đã điều trị khỏi. Tuy nhiên, chị B. không thực hiện các biện pháp phòng ngừa.</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -2861,12 +2861,12 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Giảm nguy cơ lây bệnh lao trong cộng đồng</t>
+          <t>Cảnh báo nguy cơ dịch chồng dịch ở phía Nam, đã có 12 ca tử vong</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Tại Việt Nam, thách thức từ lao kháng thuốc và định kiến xã hội vẫn đang là rào cản ngăn người bệnh điều trị bệnh lao tại cộng đồng. Để có thể đạt mục tiêu cơ bản chấm dứt dịch bệnh lao vào năm 2030, ngành y tế cần tăng cường khám sàng lọc, phát hiện sớm bệnh lao, từ đó nâng cao hiệu quả điều trị, nhất là giảm nguy cơ lây lan trong cộng đồng.</t>
+          <t>Ngày 14-4, trước tình hình dịch bệnh tay chân miệng (TCM) và sốt xuất huyết (SXH) đang gia tăng, lãnh đạo Cục Phòng bệnh, Bộ Y tế đã thông tin về diễn biến 2 dịch bệnh truyền nhiễm này và các biện pháp ứng phó của ngành y tế.</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -2883,12 +2883,12 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Pháp phong tỏa tàu chở hơn 1.700 người sau ca tử vong nghi do nhiễm virus</t>
+          <t>Số ca tay chân miệng và sốt xuất huyết gia tăng, đã có 12 người tử vong</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Pháp phong tỏa tàu chở hơn 1.700 người sau ca tử vong nghi do nhiễm virus</t>
+          <t>(PLO)- Cả nước ghi nhận hàng chục ngàn ca mắc tay chân miệng và sốt xuất huyết với 12 trường hợp tử vong, ngành y tế khuyến cáo người dân chủ động triển khai các biện pháp phòng dịch.</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -2905,12 +2905,12 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Điều tra: Thịt bẩn luồn lách đến bữa ăn - Kỳ 1: Thâm nhập lò mổ heo chết</t>
+          <t>Bệnh viêm não mô cầu, tay chân miệng diễn biến phức tạp ở ĐBSCL</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>(PLO)- Từ những con heo chết, PV ghi nhận một lò mổ hoạt động xuyên đêm, nơi thịt được xẻ ra, đóng thùng và nhanh chóng đưa đi tiêu thụ.</t>
+          <t>Bệnh viêm não mô cầu ghi nhận thêm một ca tử vong, trong khi số ca mắc tay chân miệng tăng 2,5 lần so với cùng kỳ 2025.</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -2920,19 +2920,19 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Bộ Y tế thông tin về chủng vi rút Hanta đang được WHO cảnh báo</t>
+          <t>Gần 32.000 ca mắc sốt xuất huyết: Cảnh báo số ca mắc có thể tăng mạnh</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Trước các thông tin quốc tế liên quan đến chùm ca bệnh do vi rút Hanta ghi nhận trên tàu du lịch quốc tế MV Hondius, ngày 13-5, Cục Phòng bệnh Bộ Y tế có văn bản khẩn thông tin về tình hình dịch bệnh và khuyến cáo.</t>
+          <t>Từ đầu năm 2026 đến nay, cả nước ghi nhận 31.927 ca mắc sốt xuất huyết, trong đó có 4 trường hợp tử vong.  Trong bối cảnh thời tiết nóng ẩm đến sớm, mưa thất thường và điều kiện sinh hoạt thuận lợi cho muỗi phát triển, ngành y tế cảnh báo số ca mắc có thể tiếp tục gia tăng trong thời gian tới</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -2949,12 +2949,12 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Chùm ca nhiễm virus Hanta trên tàu du lịch: Bộ Y tế phát khuyến cáo khẩn</t>
+          <t>Nắng nóng, bệnh viện quá tải vì nhiều người già và trẻ em bị ốm</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>(NLĐO) - Chùm ca nhiễm virus Hanta trên tàu MV Hondius khiến 3 người tử vong, Bộ Y tế khuyến cáo người dân theo dõi sức khỏe, chủ động phòng chống chuột.</t>
+          <t>TPO - Nắng nóng gay gắt kèm gió Lào khiến Nghệ An có thời điểm lên tới hơn 40°C, kéo theo số ca nhập viện tăng mạnh, đặc biệt là người già và trẻ nhỏ.</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -2971,12 +2971,12 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Việt Nam chưa ghi nhận ca mắc virus Hanta</t>
+          <t>Tay chân miệng tăng nhanh, Bộ Y tế khuyến cáo cho trẻ nghỉ học khi mắc bệnh</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Chiều 13-5, Cục Phòng bệnh (Bộ Y tế) có công văn khẩn gửi các đơn vị chức năng của Bộ Y tế cập nhật thông tin về chùm ca bệnh do virus Hanta gây ra trên tàu du lịch quốc tế MV Hondius khi đang trên hành trình từ Argentina tới Cape Verde (quốc đảo ngoài khơi Tây Phi).</t>
+          <t>Tay chân miệng tăng nhanh, Bộ Y tế khuyến cáo cho trẻ nghỉ học khi mắc bệnh</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -2993,12 +2993,12 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Khám sàng lọc lao cho người dân tại vùng cao</t>
+          <t>Chủng EV71 gây bệnh nặng lưu hành, tay chân miệng đối mặt nguy cơ bùng phát mạnh</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Các bác sĩ Bệnh viện Phổi Trung ương vừa thực hiện gần 2.000 lượt khám sàng lọc lao cho người dân tại vùng cao, qua đó kịp thời phát hiện bệnh lao cũng như các bệnh lý khác để đưa vào điều trị, cũng như bảo vệ cộng đồng khỏi nguồn lây.</t>
+          <t>TPO - Bệnh tay chân miệng đang gia tăng tại nhiều địa phương, nhất là phía Nam, với hàng chục nghìn ca mắc và sự lưu hành của chủng EV71 nguy cơ gây bệnh nặng. Ngành y tế cảnh báo dịch có thể tiếp tục diễn biến phức tạp nếu không triển khai đồng bộ các biện pháp phòng, chống. Ông Võ Hải Sơn, Phó Cục trưởng Cục phòng bệnh (Bộ Y tế) trao đổi với báo chí xung quanh dịch bệnh này.</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -3015,12 +3015,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Hantavirus dễ nhầm với cúm có thể chuyển nặng nhanh</t>
+          <t>4 người chết do não mô cầu, Bộ Y tế khẩn cấp khuyến cáo</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Một chùm ca nhiễm Hantavirus xuất hiện trên tàu du lịch quốc tế với 3 trường hợp tử vong đang khiến giới y tế toàn cầu lo ngại. Bệnh có biểu hiện ban đầu rất dễ nhầm với cúm.</t>
+          <t>TPO - Ngày 13/4, Bộ Y tế cho biết từ đầu năm đến nay, cả nước ghi nhận 24 trường hợp mắc bệnh do não mô cầu, trong đó có 4 ca tử vong. Số ca mắc đang có xu hướng gia tăng hơn so với cùng kì năm 2025 cho thấy nguy cơ bệnh diễn biến phức tạp, tỉ lệ tử vong cao.</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -3037,12 +3037,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>3 người tử vong trên tàu du lịch Hà Lan, Bộ Y tế khuyến cáo phòng bệnh từ chuột</t>
+          <t>Số ca não mô cầu tăng so với cùng kỳ, Bộ Y tế khuyến cáo cộng đồng chủ động phòng bệnh</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Trước thông tin về chùm ca bệnh do virus Hanta trên tàu du lịch Hà Lan, Cục Phòng bệnh (Bộ Y tế)  khuyến cáo người dân chủ động phòng bệnh, đặc biệt trong bối cảnh chuột phổ biến tại nhiều địa phương.</t>
+          <t>Bộ Y tế cho biết, hiện số trường hợp mắc bệnh não mô cầu có xu hướng gia tăng trong thời gian gần đây và cao hơn so với cùng kỳ năm 2025, trong đó có 4 trường hợp tử vong.</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -3059,12 +3059,12 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Phòng, chống virus Hanta: Việt Nam tăng cường giám sát tại cửa khẩu, cơ sở khám bệnh, chữa bệnh</t>
+          <t>Phát hiện 24 ca não mô cầu, đã có 4 người tử vong</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Bộ Y tế cho biết, hiện chưa ghi nhận công dân Việt Nam có liên quan đến chùm ca bệnh nhiễm virus Hanta. Cục Phòng bệnh đã có văn bản đề nghị các địa phương tăng cường giám sát tại cửa khẩu, giám sát tại cơ sở khám bệnh, chữa bệnh.</t>
+          <t>(PLO)- Số ca mắc não mô cầu có xu hướng gia tăng, trong đó ghi nhận nhiều trẻ em dưới 15 tuổi mắc bệnh và đã có những trường hợp tử vong.</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -3081,12 +3081,12 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>3 người tử vong vì virus Hanta trên tàu du lịch, Việt Nam có nguy cơ?</t>
+          <t>CDC Cà Mau khuyến cáo sau khi ghi nhận 3 ca nghi viêm não mô cầu</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>3 người tử vong vì virus Hanta trên tàu du lịch, Việt Nam có nguy cơ?</t>
+          <t>(NLĐO) – Giám đốc CDC Cà Mau Trần Hiến Khóa đã có những chia sẻ quan trọng khi địa phương ghi nhận 3 ca nghi viêm não mô cầu.</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -3103,12 +3103,12 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Phân biệt virus Hanta với cúm thường: Khi nào cần đi viện gấp?</t>
+          <t>TPHCM yêu cầu các bệnh viện sẵn sàng cách ly người nghi ngờ mắc virus Ebola</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>SKĐS - Virus Hanta đang gây chú ý sau chùm ca bệnh nghiêm trọng trên tàu du lịch quốc tế năm 2026. Bệnh lây ra sao, triệu chứng thế nào và Việt Nam có nguy cơ không?</t>
+          <t>Trước diễn biến phức tạp của dịch Ebola tại các nước châu Phi, Sở Y tế TPHCM yêu cầu toàn ngành y tế tăng cường giám sát, kích hoạt phương án phòng chống dịch...</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -3118,19 +3118,19 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Cách ly 42 ngày với người nguy cơ cao nhiễm virus Hanta</t>
+          <t>TPHCM yêu cầu các bệnh viện sẵn sàng sàng lọc, cách ly người nghi ngờ mắc bệnh do virus Ebola</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Với người tiếp xúc nguy cơ cao nhiễm virus Hanta, Tổ chức Y tế thế giới WHO khuyến cáo theo dõi chủ động và cách ly 42 ngày.</t>
+          <t>Ngày 21-5, Sở Y tế TPHCM có văn bản khẩn gửi các cơ sở y tế trên địa bàn về việc tăng cường giám sát, phòng chống nguy cơ xâm nhập bệnh do virus Ebola trên địa bàn.</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -3147,12 +3147,12 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>WHO cảnh báo chùm ca virus Hanta gây tử vong, Việt Nam tăng cường giám sát</t>
+          <t>Chuyên gia cảnh báo nguy cơ dịch bệnh do muỗi truyền, người dân không được chủ quan</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Cục Phòng bệnh (Bộ Y tế) vừa phát công văn khẩn về bệnh do virus Hanta gây ra sau khi WHO ghi nhận chùm 11 ca bệnh trên tàu MV Hondius, trong đó có 3 ca tử vong.</t>
+          <t>SKĐS - Trước nguy cơ gia tăng các bệnh do muỗi truyền trong mùa nắng nóng, chuyên gia cảnh báo người dân không được chủ quan với sốt xuất huyết, viêm não Nhật Bản hay sốt rét. Biện pháp hiệu quả nhất hiện nay vẫn là diệt lăng quăng, bọ gậy và phòng chống muỗi từ sớm.</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -3169,12 +3169,12 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Sốc sốt xuất huyết, bệnh nhi 10 tuổi suy đa cơ quan, tổn thương gan cấp tính nguy kịch</t>
+          <t>Australia chi hơn 7 triệu AUD ứng phó với bệnh bạch hầu</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>SKĐS - Mới đây, Bệnh viện Nhi đồng 1 đã tiếp nhận và điều trị thành công cho một bé gái 10 tuổi mắc sốc sốt xuất huyết Dengue nặng, tổn thương gan cấp tính.</t>
+          <t>Ngày 21/5, Bộ trưởng Y tế Australia Mark Butler thông báo về việc chính phủ nước này quyết định chi 7,2 triệu AUD để hỗ trợ Vùng lãnh thổ Bắc Australia và cộng đồng người bản địa ứng phó với dịch bệnh bạch hầu. Trong đó 5,2 triệu AUD sẽ được dùng để cử thêm các chuyên gia y tế đến tiêm vaccine phòng bệnh bạch hầu, tham gia công tác chữa bệnh và cung cấp thêm kháng sinh đến khu vực này. 2 triệu AUD còn lại sẽ được Cơ quan kiểm soát dịch bệnh của người bản địa dùng để hỗ trợ công tác thông tin, tu</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -3191,12 +3191,12 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Bệnh viện Hà Lan cách ly 12 nhân viên sau sự cố virus Hanta</t>
+          <t>Sốt xuất huyết gia tăng, nhiều phường xã tăng cường chống dịch</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Bệnh viện Hà Lan cách ly 12 nhân viên sau sự cố virus Hanta</t>
+          <t>TPHCM đã bắt đầu vào mùa mưa, sốt xuất huyết (SXH) có xu hướng gia tăng do thời tiết thuận lợi cho muỗi truyền bệnh sinh sản và phát triển. Trước bối cảnh đó, nhiều trạm y tế xã, phường, đặc khu trên địa bàn đã khẩn trương triển khai đồng bộ nhiều biện pháp ứng phó, nhằm chủ động phòng chống.</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -3213,12 +3213,12 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Nhiều nước ghi nhận ca nhiễm virus Hanta liên quan tàu MV Hondius</t>
+          <t>Bác sĩ lưu ý phòng bệnh tay chân miệng, sốt xuất huyết và não mô cầu trong mùa hè</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Nhiều nước ghi nhận ca nhiễm virus Hanta liên quan tàu MV Hondius</t>
+          <t>Chuyên gia y tế cho biết, mùa hè với thời tiết nóng ẩm là điều kiện thuận lợi để nhiều bệnh truyền nhiễm ở trẻ nhỏ gia tăng như sốt xuất huyết, tay chân miệng hay viêm não mô cầu.</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -3228,19 +3228,19 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Biến chứng thủy đậu, bé trai 6 tuổi nhiễm khuẩn huyết, phải thở máy nguy kịch</t>
+          <t>Nỗ lực kiểm soát dịch bệnh sốt xuất huyết</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>SKĐS - Tin từ Bệnh viện Bệnh Nhiệt đới Trung ương, khoa Nhi của bệnh viện đang điều trị cho bệnh nhi 6 tuổi trong tình trạng rất nặng sau biến chứng thủy đậu.</t>
+          <t>Bệnh sốt xuất huyết hiện lưu hành tại hơn 100 quốc gia, trong đó các khu vực châu Mỹ, Đông Nam Á và Tây Thái Bình Dương bị ảnh hưởng nghiêm trọng nhất, đặc biệt khu vực châu Á. Để chủ động phòng, chống dịch bệnh tại cộng đồng, Hiệp hội các quốc gia Đông Nam Á (ASEAN) và Tổ chức Y tế Thế giới chọn ngày 15/6 hằng năm là “Ngày ASEAN phòng, chống sốt xuất huyết”.</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -3257,12 +3257,12 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Vaccine cúm mùa 2026 và sự biến đổi của virus cúm: Những thông tin cần biết</t>
+          <t>Nhiều ca não mô cầu biến chứng, chuyên gia cảnh báo</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Diễn biến phức tạp của virus cúm trong thời gian cuối năm 2025, đầu năm 2026 đang đặt ra yêu cầu cấp thiết về phòng bệnh chủ động. Các chuyên gia nhấn mạnh, tiêm vaccine cúm là giải pháp hiệu quả giúp giảm thiểu nguy cơ mắc bệnh cũng như các biến chứng nghiêm trọng.</t>
+          <t>Nhiều ca não mô cầu biến chứng, chuyên gia cảnh báo</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -3279,12 +3279,12 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Manh mối dịch tễ về "bệnh nhân số 0" trong ổ dịch Hanta ở du thuyền hạng sang</t>
+          <t>Virus hợp bào hô hấp: Mối nguy khó lường với trẻ dưới 1 tuổi</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Theo New York Post, "bệnh nhân số 0" trong vụ bùng phát virus Hanta trên tàu du lịch đã được xác định là nhà điểu học người Hà Lan Leo Schilperoord (70 tuổi). Ông và vợ là bà Mirjam Schilperoord (69 tuổi) đều là những gương mặt quen thuộc trong cộng đồng nghiên cứu chim tại châu Âu.</t>
+          <t>Virus hợp bào hô hấp: Mối nguy khó lường với trẻ dưới 1 tuổi</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -3301,12 +3301,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Một phụ nữ nhiễm bệnh nguy kịch, Pháp siết chặt kiểm soát virus Hanta</t>
+          <t>Một trường hợp tử vong do vi rút hanta tại Mỹ</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Tổng thống Pháp Emmanuel Macron ngày 12/5 khẳng định tình hình liên quan đến virus Hanta tại Pháp vẫn “nằm trong tầm kiểm soát” của chính phủ, trong bối cảnh một phụ nữ Pháp nhiễm bệnh đang trong tình trạng nguy kịch và nhiều nước châu Âu tăng cường các biện pháp phòng dịch.</t>
+          <t>Giới chức y tế bang Colorado, Mỹ thông tin về một ca tử vong do vi rút hanta, cho biết giai đoạn này là thời điểm dễ ghi nhận các ca nhiễm.</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -3323,12 +3323,12 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Du thuyền có khách nhiễm vi rút Hanta hoàn tất sơ tán</t>
+          <t>TPHCM kích hoạt 'lá chắn' ngăn Ebola xâm nhập</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Reuters ngày 12.5 dẫn thông báo của nhà điều hành Oceanwide Expeditions (Hà Lan) cho hay du thuyền MV Hondius đã khởi hành từ Tây Ban Nha về Hà Lan với 25 thành viên thủy thủ đoàn cùng 1 bác sĩ và 1 điều dưỡng. Tất cả hành khách đã được sơ tán sau khi ổ dịch vi rút Hanta bùng phát trên du thuyền.</t>
+          <t>TPO - Trước diễn biến phức tạp của dịch Ebola tại châu Phi, TP.HCM đã nâng mức cảnh giác, tăng cường giám sát y tế tại sân bay, cảng biển và cửa khẩu quốc tế nhằm phát hiện sớm và xử lý ngay các trường hợp nghi ngờ để bảo vệ cộng đồng.</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -3338,19 +3338,19 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Ukraine nêu điểm yếu khiến nhiều robot thất thế ngay lần đầu xung trận</t>
+          <t>Hong Kong (Trung Quốc) kích hoạt ứng phó khẩn cấp trước dịch Ebola</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Ukraine nêu điểm yếu khiến nhiều robot thất thế ngay lần đầu xung trận</t>
+          <t>Tính đến thời điểm hiện tại, Hong Kong chưa xác nhận trường hợp nhiễm Ebola nào. Tác động tức thời của Ebola đối với sức khỏe người dân Hong Kong cũng được đánh giá là ở mức thấp. Tuy nhiên, chính quyền đặc khu này vẫn thực hiện một loạt các biện pháp phòng ngừa và kiểm soát để ngăn chặn nghiêm ngặt dịch bệnh xâm nhập.</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -3360,19 +3360,19 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>irrelevant</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Sơ tán sau 3 ca tử vong vì vi rút Hanta, tàu MV Hondius lên đường về Hà Lan</t>
+          <t>TPHCM: Kiểm soát chặt cửa khẩu chặn nguy cơ dịch bệnh Ebola xâm nhập</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Tàu MV Hondius rời Tây Ban Nha, hướng về Hà Lan. Một số hành khách tiếp tục có kết quả dương tính với vi rút Hanta sau khi hồi hương.</t>
+          <t>Ngày 19-5, Sở Y tế TPHCM cho biết, ngành y tế thành phố đang tăng cường và siết chặt công tác giám sát dịch bệnh Ebola tại các cửa khẩu nhằm chủ động phát hiện sớm, ngăn chặn nguy cơ dịch bệnh xâm nhập vào thành phố.</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -3382,19 +3382,19 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Hà Lan cách ly 12 nhân viên y tế sau sự cố xử lý ca nhiễm virus Hanta</t>
+          <t>Nhiều người Mỹ nghi nhiễm virus Ebola tại CHDC Congo</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Vụ việc xảy ra tại bệnh viện Radboudumc ở thành phố Nijmegen, nơi tiếp nhận một hành khách từ tàu du lịch MV Hondius vào ngày 7/5. Theo thông báo của bệnh viện, máu và nước tiểu của bệnh nhân đã được xử lý mà không thực hiện đầy đủ các quy trình an toàn nghiêm ngặt, dẫn đến việc 12 nhân viên y tế phải cách ly phòng ngừa trong thời gian 6 tuần.</t>
+          <t>SKĐS - Ít nhất 6 người Mỹ đã tiếp xúc với virus Ebola tại Cộng hòa Dân chủ Congo, trong đó có 3 trường hợp tiếp xúc nguy cơ cao và một người xuất hiện triệu chứng.</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -3411,12 +3411,12 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Vận hành nguồn Quỹ Toàn cầu công khai, minh bạch, đúng quy định và vì lợi ích của người dân</t>
+          <t>Hơn 80 ca tử vong nghi do nhiễm virus Ebola ở Congo, Bộ Y tế ra thông báo khẩn</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>SKĐS - Chiều 12/5, tại Bộ Y tế, PGS.TS Nguyễn Thị Liên Hương, Thứ trưởng Bộ Y tế, Chủ tịch Ban điều phối Quốc gia Quỹ Toàn cầu phòng, chống AIDS, Lao và Sốt rét tại Việt Nam (CCM) chủ trì cuộc họp chuẩn bị xây dựng Hồ sơ đề xuất viện trợ Quỹ Toàn cầu, giai đoạn 2027-2029.</t>
+          <t>Tối 17-5, ngay sau khi Tổ chức Y tế thế giới (WHO) cảnh báo về dịch bệnh sốt xuất huyết do virus Ebola gây ra tại Cộng hòa Dân chủ Congo và Uganda với hơn 80 người tử vong, Bộ Y tế đã thông tin tới báo chí về các biện pháp ứng phó với dịch bệnh nguy hiểm này.</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -3426,19 +3426,19 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>noise</t>
+          <t>relevant</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Thái Lan siết chặt kiểm tra y tế tại sân bay quốc tế để ngăn chặn virus Hanta</t>
+          <t>Hơn 80 ca tử vong nghi do nhiễm virus Ebola ở Congo, Bộ Y tế ra thông báo khẩn</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Cục trưởng DDC, Tiến sĩ Montien Kanasawadse, cho biết quyết định tăng cường quy trình sàng lọc sức khỏe đối với hành khách nhập cảnh từ các quốc gia và vùng lãnh thổ Nam Mỹ tại các sân bay quốc tế lớn, vừa để trấn an công chúng, vừa khẳng định chính phủ đã triển khai đầy đủ các bước phòng ngừa cần thiết, dù đến nay chưa ghi nhận ca nhiễm virus Hanta nào tại Thái Lan. Ông Montien nhấn mạnh, động thái này cũng nhằm bảo đảm môi trường du lịch an toàn.</t>
+          <t>Tối 17-5, ngay sau khi Tổ chức Y tế thế giới (WHO) cảnh báo về dịch bệnh sốt xuất huyết do virus Ebola gây ra tại Cộng hòa Dân chủ Congo và Uganda với hơn 80 người tử vong, Bộ Y tế đã thông tin tới báo chí về các biện pháp ứng phó với dịch bệnh nguy hiểm này.</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -3455,12 +3455,12 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Bé trai 6 tuổi nguy kịch vì biến chứng nặng từ thủy đậu</t>
+          <t>WHO: Nguy cơ bùng phát virus Hanta vẫn thấp</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>TPO - Từ những nốt phỏng nước tưởng chừng thông thường do thủy đậu, một bé trai 6 tuổi ở Lai Châu đã rơi vào tình trạng nguy kịch với suy hô hấp nặng, nhiễm khuẩn huyết do phế cầu và phải thở máy xâm nhập.</t>
+          <t>Tổ chức Y tế thế giới (WHO) thông báo vẫn giữ nguyên mức đánh giá nguy cơ thấp đối với đợt bùng phát virus Hanta trên một con tàu du lịch đang tiến về Hà Lan.</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -3469,6 +3469,1392 @@
         </is>
       </c>
       <c r="D139" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>WHO: Đợt bùng phát virus Hanta 'nguy cơ thấp'</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Tổ chức Y tế Thế giới (WHO) ngày 17/5 tuyên bố vẫn giữ nguyên đánh giá đợt bùng phát virus Hanta ở mức "nguy cơ thấp" khi con tàu du lịch khởi phát dịch bệnh này đang tiến gần đến Hà Lan.</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Điểm đáng lo ngại của dịch Ebola đang bùng phát tại châu Phi</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Theo Tổ chức Y tế Thế giới (WHO), đây mới là lần thứ ba chủng virus Bundibugyo được phát hiện, dù trước đó đã có hơn 20 đợt bùng phát Ebola tại Congo và Uganda. Đợt bùng phát hiện nay được xác nhận vào ngày 15/5 vừa qua. Tổ chức Y tế Thế giới đã ban bố tình trạng khẩn cấp y tế công cộng quốc tế sau khi ghi nhận hơn 300 ca nghi nhiễm và 88 ca tử vong liên quan đến dịch bệnh này.</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Ebola ở Congo, Uganda thành tình trạng khẩn cấp quốc tế, Bộ Y tế phát khuyến cáo</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>WHO xác định đợt bùng phát Ebola chủng Bundibugyo tại Cộng hòa Dân chủ Congo và Uganda là “sự kiện y tế công cộng khẩn cấp gây quan ngại quốc tế”. Bộ Y tế Việt Nam khẳng định chưa ghi nhận dịch lan rộng toàn cầu, đồng thời tăng cường giám sát, kiểm dịch và khuyến cáo người dân theo dõi sức khỏe khi trở về từ vùng dịch.</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Pháp tuyên bố chủng virus hanta trên du thuyền MV Hondius trùng khớp với chủng đã biết</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>SKĐS - Viện Pasteur của Pháp đã giải trình tự hoàn chỉnh virus hanta phát hiện ở hành khách người Pháp trên du thuyền MV Hondius và xác nhận chủng virus này hoàn toàn trùng khớp với các chủng đã biết.</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>WHO tuyên bố dịch Ebola là tình trạng khẩn cấp toàn cầu</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>SKĐS - WHO đã chính thức tuyên bố dịch Ebola do chủng virus Bundibugyo gây ra là tình trạng khẩn cấp về sức khỏe công cộng quốc tế, chỉ một ngày sau khi dịch bệnh bùng phát tại CHDC Congo và Uganda.</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Cà Mau: Một trường hợp tử vong nghi mắc viêm não mô cầu</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Ngày 10-4, thông tin từ Trung tâm Kiểm soát bệnh tật tỉnh Cà Mau cho biết, trên địa bàn ấp 6 (xã Khánh An, tỉnh Cà Mau) vừa ghi nhận 3 trường hợp nghi mắc viêm não mô cầu, trong đó có 1 trường hợp đã tử vong.</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Cà Mau: Một ca tử vong nghi viêm não mô cầu</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Chiều 10-4, thông tin từ Trung tâm Kiểm soát bệnh tật tỉnh Cà Mau (CDC Cà Mau) trên địa bàn đã ghi nhận các trường hợp nghi mắc bệnh viêm màng não do não mô cầu gây ra, trong đó đã có 1 người tử vong.</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Cà Mau báo cáo 3 người nghi mắc não mô cầu,1 trường hợp đã tử vong</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>TPO - Ba trường hợp nghi mắc viêm não mô cầu được phát hiện tại ấp 6, xã Khánh An, tỉnh Cà Mau, trong số đó 1 ca đã tử vong. Tất cả trong số này đều trên 30 tuổi.</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Cà Mau ghi nhận 3 trường hợp nghi viêm não mô cầu, 1 người tử vong</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>(NLĐO) - Ngành y tế Cà Mau đang triển khai các biện pháp giám sát, xử lý ổ dịch để ngăn chặn nguy cơ lây lan trong cộng đồng.</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Cà Mau ghi nhận 3 ca nghi viêm não mô cầu, 1 trường hợp tử vong</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Ba trường hợp nghi mắc viêm não mô cầu được phát hiện tại ấp 6, xã Khánh An, tỉnh Cà Mau; trong đó  có 1 ca tử vong. Ngành y tế đang khẩn trương kích hoạt giám sát, xử lý dịch tễ diện rộng.</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Căn bệnh nguy hiểm diễn tiến tối cấp, trở nặng chỉ trong vài giờ</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Căn bệnh nguy hiểm diễn tiến tối cấp, trở nặng chỉ trong vài giờ</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Xuất hiện ổ dịch sốt xuất huyết đầu tiên tại Hà Tĩnh trong năm 2026</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Hiện nay tại Hà Tĩnh ghi nhận 4 trường hợp mắc dịch sốt xuất huyết Dengue, đây là ổ dịch đầu tiên được phát hiện kể từ đầu năm đến nay. Ngành y tế địa phương đang triển khai các biện pháp khẩn cấp để khoanh vùng ổ dịch.</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Đắk Lắk liên tiếp phát hiện các ổ dịch bệnh truyền nhiễm</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>3 trường hợp mắc quai bị đầu tiên được phát hiện vào ngày 6/4 tại Trường Tiểu học Trần Văn Ơn, phường Buôn Ma Thuột, Đắk Lắk. Qua rà soát mở rộng, nhà trường phát hiện thêm 8 trường hợp có cùng triệu chứng sốt, sưng đau vùng mang tai, khó nhai nuốt và mệt mỏi. Cũng trong ngày 6/4, tại Trường Tiểu học Lê Văn Tám, phường Buôn Ma Thuột ngành y tế ghi nhận 9 ca mắc khác, nâng tổng số ca mắc lên 12 bệnh nhân. Ngay sau khi phát hiện các ca bệnh, Trạm Y tế phường Buôn Ma Thuột đã báo cáo Sở Y tế tỉnh Đ</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Người dân chủ động phòng ngừa nhiễm biến thể mới Covid-19 Ve sầu</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>SKĐS - Thông tin về biến thể mới của COVID-19 đang thu hút sự quan tâm của nhiều người dân. Tại Nghệ An, dù chưa ghi nhận ca mắc liên quan biến thể BA3.2 (còn gọi là Ve sầu), tâm lý lo lắng trước nguy cơ dịch bệnh quay trở lại là điều khó tránh khỏi.</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>U.S. Health Officials Confirm Four New Bird Flu Cases</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Earlier this year the virus, known as H5N1 , was detected in U.S. livestock, and is now circulating in cattle in several states.</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>H5N1 bird flu spreads to sea otters and sea lions along San Mateo coast, wildlife experts say - AOL</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>After H5N1 bird flu was detected in elephant seals gathered at Año Nuevo State Park, other marine mammals have also succumbed, including a sea ...</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Ano Nuevo preserve to reopen after bird flu outbreak kills elephant seals - CBS News</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>H5N1 strains have been linked to severe illness and widespread mortality in marine mammals in other parts of the world. While the risk of infection to ...</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Top Cardiovascular Organizations Join Forces for International Scientific - Bioengineer.org</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>By elucidating novel therapeutics, optimizing procedural strategies, and exploring emerging disease intersections such as COVID-19, the summit ...</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Ca tay chân miệng TP HCM tăng hơn 60%</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>TP HCM ghi nhận thêm 1.347 ca mắc tay chân miệng trong tuần qua, tăng 64% so với trung bình 4 tuần trước, nâng tổng số bệnh nhân từ đầu năm vượt 10.000.</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Local Landscaper Tackles the Hamptons Bird Flu Problem - The New York Times</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Their deaths came at a time when much of the North Fork of Long Island was hit with a scourge of H5N1 , also known as bird flu. Wildlife ...</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Hà Tĩnh xuất hiện ổ dịch sốt xuất huyết Dengue</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Ngày 8-4, ông Nguyễn Chí Thanh, Giám đốc Trung tâm Kiểm soát bệnh tật (CDC) tỉnh Hà Tĩnh cho biết, từ ngày 3-4 đến nay, tại tổ dân phố Hợp Tiến, phường Vũng Áng đã xuất hiện 4 trường hợp mắc sốt xuất huyết Dengue. Đây là ổ dịch sốt xuất huyết Dengue đầu tiên trên địa bàn tỉnh từ đầu năm đến nay.</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Virus viêm gan B có lây qua dịch đàm nhớt?</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Virus viêm gan B có lây qua dịch đàm nhớt không? Nên phòng ngừa thế nào khi tiếp xúc người mắc viêm gan B và bệnh hô hấp? (Trần Thị Mến, 22 tuổi, Sơn La)</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Sốt xuất huyết: phát hiện sớm để tránh biến chứng</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Khởi đầu chỉ là một cơn sốt cao, mệt mỏi như cúm thông thường nhưng chỉ sau 2-3 ngày, sốt xuất huyết có thể chuyển nặng, tấn công vào các tế bào máu và nhiều cơ quan nội tạng. “Đại dịch ngồi” đẩy người trẻ vào nguy cơ liệt: Cảnh báo từ ca bệnh điển hình Hút thuốc lá làm "bóp nghẹt" mạch máu khi chơi thể thao Từ móng giò đến rau xanh: Lời khuyên dinh dưỡng cho sản phụ [Video] Tăng nguy cơ đột tử khi chơi thể thao vì thói quen này 1000 ca cấp cứu Tết: Khi hệ thống cấp cứu được "thử thách" phản ứng...</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Hà Tĩnh xuất hiện ổ dịch sốt xuất huyết Dengue</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Ngày 8-4, ông Nguyễn Chí Thanh, Giám đốc Trung tâm Kiểm soát bệnh tật (CDC) tỉnh Hà Tĩnh cho biết, từ ngày 3-4 đến nay, tại tổ dân phố Hợp Tiến, phường Vũng Áng đã xuất hiện 4 trường hợp mắc sốt xuất huyết Dengue. Đây là ổ dịch sốt xuất huyết Dengue đầu tiên trên địa bàn tỉnh từ đầu năm đến nay. Xuất hiện ổ dịch sốt xuất huyết Dengue đầu tiên tại Hà Tĩnh Dịch bệnh sốt xuất huyết và tay chân miệng tăng rất cao, Bộ Y tế chỉ đạo khẩn Hà Tĩnh: Khống chế thành công ổ dịch sốt xuất huyết Dengue</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Hà Tĩnh xuất hiện ổ dịch sốt xuất huyết</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>SKĐS - Sau khi có thông tin về trường hợp mắc sốt xuất huyết, các lực lượng chức năng tỉnh Hà Tĩnh triển khai các biện pháp phòng, chống dịch nhằm không để lây lan ra diện rộng. Đồng thời tiến hành điều tra các ca bệnh nghi ngờ sốt xuất huyết, lấy máu xét nghiệm.</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Life at SLO County elephant seal beach goes on despite threat of bird flu - PressReader</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>A complication this year is the threat of H5N1 , Highly Pathogenic Avian Influenza, which hangs over them. The outbreak has been confined to San Mateo ...</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Tay chân miệng vào mùa dễ lây lan, nhận diện nguy cơ và cách phòng bệnh cho trẻ</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>SKĐS - Trước tình trạng số ca tay chân miệng tăng so với cùng kỳ, ngành y tế Huế khuyến cáo chủ động nhận diện yếu tố nguy cơ, tăng cường vệ sinh và thực hiện các biện pháp phòng bệnh.</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Đắk Lắk chủ động kiểm soát dịch bệnh ở trẻ em</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>VOV.VN - Trong bối cảnh các bệnh tay chân miệng, thủy đậu và sốt xuất huyết ở trẻ em gia tăng, tiềm ẩn nguy cơ bùng phát dịch trên diện rộng, ngành y tế Đắk Lắk đang khẩn trương triển khai đồng bộ các giải pháp kiểm soát tình hình.</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Bird flu spreads across four districts in Nepal - Social News XYZ</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Kathmandu, April 7 (SocialNews.XYZ) The H5N1 highly pathogenic avian influenza, also commonly called bird flu, has spread across four districts of ...</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Bird flu spreads across four districts in Nepal - The Hans India</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Kathmandu: The H5N1 highly pathogenic avian influenza, also commonly called bird flu, has spread across four districts of Nepal, a government ...</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Cảnh báo biến thể của EV71 gây tay chân miệng rất nguy hiểm, né miễn dịch</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>(Dân trí) - Bác sĩ cảnh báo, điểm đáng ngại nhất trong tình hình bệnh tay chân miệng hiện nay là sự xuất hiện của biến thể C1 với độc lực cao và khả năng né miễn dịch, gây nguy cơ lớn cho trẻ.</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>9 học sinh một trường tiểu học ở Đắk Lắk mắc quai bị</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Tại một trường tiểu học trên địa bàn tỉnh Đắk Lắk có 9 học sinh từ lớp 1 đến lớp 3 mắc bệnh quai bị. Phát hiện ổ dịch thuỷ đậu tại một điểm trường tiểu học ở Đắk Lắk Một xã ở Phú Thọ ghi nhận 45 ca mắc sởi, ổ dịch tập trung ở trường học</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Đắk Lắk: Ghi nhận các ổ dịch quai bị và thủy đậu trong trường học</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Ngày 4-4, Trung tâm Y tế Krông Búk, tỉnh Đắk Lắk cho biết, vừa ghi nhận một ổ dịch bệnh quai bị tại Trường Tiểu học Phạm Hồng Thái (xã Cư Pơng, tỉnh Đắk Lắk).</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Đắk Lắk: Ghi nhận các ổ dịch quai bị và thủy đậu trong trường học</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Ngày 4-4, Trung tâm Y tế Krông Búk, tỉnh Đắk Lắk cho biết, vừa ghi nhận một ổ dịch bệnh quai bị tại Trường Tiểu học Phạm Hồng Thái (xã Cư Pơng, tỉnh Đắk Lắk). Khẩn cấp ứng phó với dịch bệnh tay chân miệng Dịch bệnh sốt xuất huyết và tay chân miệng tăng rất cao, Bộ Y tế chỉ đạo khẩn</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>TPHCM có 858 ca mắc tay chân miệng trong một tuần</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>TPHCM ghi nhận số ca mắc tay chân miệng (TCM) tăng mức báo động với 858 ca mắc, tăng 66,9% so với trung bình 4 tuần trước, trong đó có một ca tử vong. Dịch bệnh sốt xuất huyết và tay chân miệng tăng rất cao, Bộ Y tế chỉ đạo khẩn Số ca mắc tay chân miệng tại TPHCM tăng cao, đã có 3 ca tử vong Số trẻ mắc tay chân miệng chuyển nặng có xu hướng gia tăng</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Đắk Lắk: Xuất hiện ổ dịch quai bị tại trường tiểu học</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>(PLO)- Chín học sinh tại một trường học ở Đắk Lắk mắc bệnh quai bị với các triệu chứng sốt, sưng đau vùng mang tai và khó nhai nuốt. 23 học sinh và giáo viên mắc thủy đậu, 1 điểm trường nghỉ học</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Phát hiện ổ dịch thuỷ đậu tại một điểm trường tiểu học ở Đắk Lắk</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Sau khi ghi nhận hàng chục học sinh và giáo viên tiểu học ở tỉnh Đắk Lắk mắc thuỷ đậu, điểm trường này đã cho học sinh tạm nghỉ học. Ngành Y tế tỉnh đã tổ chức khử khuẩn, khoanh vùng và ngăn chặn dịch bệnh lây lan. Người đàn ông nguy kịch vì lây thuỷ đậu từ con gái Vì sao bệnh tay chân miệng đang trở nên nguy hiểm và khó lường? Nhiều ca bệnh tay chân miệng tăng nặng: Bộ Y tế chỉ đạo khẩn</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Phát hiện ổ dịch thủy đậu, một điểm trường cho học sinh nghỉ học</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>(NLĐO) – Sau khi ghi nhận hàng chục học sinh và giáo viên mắc bệnh thủy đậu, ngành chức năng tỉnh Đắk Lắk đã cho học sinh tại đây nghỉ học.</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Biến thể ve sầu BA.3.2: Né miễn dịch tốt nhưng xâm nhập kém</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>(PLO)- Sự xuất hiện của biến thể ve sầu BA.3.2 gây chú ý do có nhiều đột biến. Người dân cần chủ động phòng bệnh, không hoang mang nhưng cũng không nên chủ quan. Hà Nội ghi nhận 29 ca mắc COVID-19, khuyến cáo về biến thể ve sầu BA.3.2 Biến thể BA.3.2 của COVID-19 âm thầm lan rộng, Bộ Y tế khuyến cáo Biến thể BA.3.2 của COVID-19 nguy hiểm đến mức nào?</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>25 giáo viên, học sinh một điểm trường mắc thủy đậu</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>(Dân trí) - Một ổ dịch thủy đậu được phát hiện tại một điểm trường ở Đắk Lắk khiến 23 học sinh và 3 giáo viên mắc bệnh. Ngành y tế tỉnh đã tổ chức khử khuẩn, khoanh vùng và ngăn chặn dịch bệnh lây lan.</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>23 học sinh và giáo viên mắc thủy đậu, 1 điểm trường nghỉ học</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>(PLO)- Một điểm trường ở Đắk Lắk phải cho học sinh nghỉ học vì giáo viên, học sinh bị mắc thủy đậu. Người đàn ông 36 tuổi suy hô hấp nguy kịch vì lây thủy đậu từ con</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>TPHCM ghi nhận hơn 9.100 ca mắc tay chân miệng, 6 người nhiễm não mô cầu</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>(Dân trí) - Số ca bệnh tay chân miệng ở TPHCM đã tăng 191,5% so với cùng kỳ năm 2025, đồng thời địa phương cũng ghi nhận các trường hợp nhiễm não mô cầu nguy hiểm.</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Hà Nội gia tăng bệnh nhân mắc COVID-19, cảnh báo đối tượng dễ bị tổn thương</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>SKĐS - COVID-19 là bệnh truyền nhiễm do virus gây ra, có đặc điểm liên tục biến đổi theo thời gian. Việc xuất hiện các biến thể mới trong giai đoạn hiện nay, trong đó có biến thể được gọi là “ve sầu”, là điều hoàn toàn có thể xảy ra khi virus vẫn tiếp tục lưu hành trong cộng đồng.</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>TPHCM: Số ca mắc tay chân miệng tăng 191,5%</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Bà Lê Hồng Nga, Phó Giám đốc HCDC cho biết, tính từ đầu năm đến ngày 29-3, TPHCM đã ghi nhận 9.107 ca mắc tay chân miệng, tăng 191,5% so với cùng kỳ năm 2025. Đầu tháng 3 đến nay, số ca mắc hàng tuần có xu hướng tăng liên tục.</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>TPHCM: Số ca mắc tay chân miệng tăng</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Lãnh đạo Trung tâm Kiểm soát bệnh tật TPHCM (HCDC) cho biết, tính từ đầu năm đến ngày 29-3, TPHCM ghi nhận 9.107 ca mắc, tăng 191,5% so với cùng kỳ năm 2025. TPHCM tổ chức tour trực thăng ngắm thành phố từ trên cao</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>TP.HCM: Số ca tay chân miệng tăng, trẻ dưới 5 tuổi chiếm đa số</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>(PLO)- Từ đầu năm đến nay, TP.HCM ghi nhận số ca tay chân miệng tăng nhanh, chủ yếu trẻ dưới 5 tuổi, ngành y tế khuyến cáo phòng bệnh kịp thời. Số ca mắc tay chân miệng tăng, Sở GD&amp;ĐT TP.HCM thông báo khẩn Nhận diện ‘dấu hiệu vàng’ chuyển nặng ở trẻ mắc tay chân miệng Chủng EV71 gây bệnh tay chân miệng nguy hiểm ra sao? Tay chân miệng tăng cao, nhiều ca nặng, chủng EV71 chiếm ưu thế</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Hà Nội: Chỉ vài ngày ho sốt, nhiều trẻ đã viêm phổi nặng vì RSV</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>(Dân trí) - Từ những cơn ho, sốt, khò khè tưởng chừng thông thường, nhiều trẻ nhỏ ở Hà Nội đã nhanh chóng chuyển viêm phổi, suy hô hấp vì RSV, thậm chí phải thở máy.</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Bộ Y tế phát công điện hỏa tốc về dịch tay chân miệng</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Trong bối cảnh số ca bệnh tay chân miệng đang tăng rất nhanh, chiều ngày 31/3, Bộ Y tế đã ban hành công văn hỏa tốc yêu cầu toàn hệ thống khám chữa bệnh tăng cường phân luồng, thu dung, điều trị và kiểm soát lây nhiễm nhằm hạn chế tối đa các ca bệnh nặng và tử vong, đặc biệt là tại khu vực phía Nam. Hà Nội tăng cường giám sát khi có 17 ca COVID-19, dịch tay chân miệng diễn biến phức tạp Điều trị ung thư, chạy thận không thu thêm phí ngoài BHYT tại bệnh viện tư Thai bám vào ‘tử huyệt’ khiến mẹ su...</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Gần 3.000 trẻ mắc tay chân miệng, bác sĩ cảnh báo dấu hiệu trở nặng</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Bệnh tay chân miệng đang gia tăng nhanh với gần 3.000 ca ghi nhận tại Bệnh viện Nhi Trung ương từ đầu năm đến nay.</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>3 trẻ tử vong do bệnh tay chân miệng, Sở Y tế TPHCM chỉ đạo khẩn</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Sau khi ghi nhận 3 trẻ tử vong, Sở Y tế TPHCM ban hành chỉ đạo khẩn ứng phó dịch tay chân miệng đang bùng phát với hơn 7.000 ca mắc trong 11 tuần đầu năm 2026.</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Số ca tay chân miệng tăng gấp 5 lần, 4 trẻ tử vong, Bộ Y tế chỉ đạo khẩn</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Số ca tay chân miệng tăng đột biến, chủ yếu ở trẻ nhỏ, với gần 25.000 trường hợp và 4 ca tử vong chỉ trong 3 tháng đầu năm. Bộ Y tế cảnh báo nguy cơ bùng phát dịch và yêu cầu siết chặt các biện pháp kiểm soát.</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Virus EV71 tấn công trẻ mắc tay chân miệng, gây biến chứng thần kinh nguy hiểm</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Sự xuất hiện của virus EV71 đang khiến nhiều trẻ mắc bệnh tay chân miệng có nguy cơ diễn tiến nặng chỉ trong 24 giờ, với biến chứng thần kinh nguy hiểm nếu không được phát hiện và xử trí kịp thời.</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Cảnh báo: Virus mới khiến trẻ mắc tay chân miệng chuyển nặng, tử vong rất nhanh</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Số ca tay chân miệng tại khu vực phía Nam đang gia tăng trở lại, xuất hiện nhiều trường hợp nặng, tử vong. Đáng lo ngại, không ít trẻ có biểu hiện không điển hình, dễ bị bỏ sót, khiến việc phát hiện và điều trị chậm trễ, làm tăng nguy cơ biến chứng nguy hiểm. Dịch tay chân miệng bùng phát, nhiều địa phương ‘than’ thiếu thuốc Liên tiếp 5 trẻ tử vong, nguy cơ dịch tay chân miệng bùng phát Sau ca tử vong do não mô cầu, người dân đổ xô đi tiêm vắc xin</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Hà Nội ghi nhận 29 ca mắc COVID-19, khuyến cáo về biến thể ve sầu BA.3.2</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>(PLO)- Hà Nội ghi nhận số ca COVID-19 tăng trong tháng 3 đầu năm 2026, ngành y tế khuyến cáo người dân không chủ quan, tiếp tục thực hiện biện pháp phòng dịch cơ bản. Biến thể BA.3.2 của COVID-19 âm thầm lan rộng, Bộ Y tế khuyến cáo TP.HCM kiểm tra các hoạt động liên quan đến thuốc, vaccine, mỹ phẩm, hóa chất y tế Tay chân miệng tăng cao, nhiều ca nặng, chủng EV71 chiếm ưu thế</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Hà Nội khuyến cáo người dân không hoang mang với biến thể COVID-19 mới BA.3.2</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>VOV.VN - Các chuyên gia y tế nhận định, sự xuất hiện của các biến thể mới là quy luật tiến hóa tự nhiên của virus. Vì vậy, việc duy trì hệ thống giám sát dịch tễ và nâng cao ý thức phòng bệnh trong cộng đồng tiếp tục giữ vai trò quan trọng, cần thiết.</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Ca mắc tay chân miệng tăng gấp 5 lần, 92% tập trung ở trẻ mầm non</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>VOV.VN - Số ca tay chân miệng tăng gấp 5 lần trong đầu năm 2026, trong đó hơn 92% tập trung ở trẻ mầm non, khiến nguy cơ bùng phát dịch tại trường học gia tăng. Chuyên gia cảnh báo cần siết chặt vệ sinh và phát hiện sớm “thời điểm vàng” để kiểm soát bệnh hiệu quả.</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Số ca tay chân miệng tăng mạnh, cảnh báo nguồn lây từ tay nắm cửa, đồ chơi</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>VOV.VN - Số ca tay chân miệng đang tăng mạnh tại nhiều địa phương, đặc biệt ở TP.HCM, với nguy cơ lây lan cao từ tay bẩn, đồ chơi, tay nắm cửa và các bề mặt sinh hoạt quen thuộc, khiến trẻ nhỏ dễ mắc bệnh nếu chủ quan phòng ngừa.</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Bộ Y tế theo dõi chặt chẽ biến thể &amp;apos;ve sầu&amp;apos; của virus SASR-CoV-2</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Theo Bộ Y tế, biến thể virus SARS-CoV-2 BA.3.2 của Covid-19 với số lượng đột biến lớn và khả năng né miễn dịch đang âm thầm lan rộng tại Mỹ và nhiều quốc gia.</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Bộ Y tế ra khuyến cáo về biến thể mới của SARS-CoV-2</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Sáng 29/3 Bộ Y tế cho biết biến thể SARS-CoV-2 là BA.3.2 được Tổ chức Y tế Thế giới xếp vào nhóm theo dõi với nguy cơ thấp. Bộ Y tế cho biết đang tiếp tục giám sát chặt chẽ, khuyến cáo người dân không chủ quan nhưng cũng không hoang mang trước diễn biến mới của dịch bệnh. Sau ca tử vong do não mô cầu, người dân đổ xô đi tiêm vắc xin Cảnh báo xu hướng trẻ hóa bệnh ung thư thực quản Việt Nam chính thức phê duyệt kỹ thuật hồi sinh tim phổi bằng tuần hoàn ngoài cơ thể</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Nhiều người lớn nguy kịch vì mắc bệnh thường gặp ở trẻ nhỏ</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Ghi nhận tại Bệnh viện Bệnh Nhiệt đới Trung ương và Bệnh viện Bạch Mai cho thấy, thời gian gần đây số ca người trưởng thành mắc thủy đậu có biến chứng nặng đang gia tăng. Không còn là bệnh “lành tính” như quan niệm phổ biến, thủy đậu ở người lớn có thể diễn tiến nhanh, dẫn tới sốc nhiễm khuẩn, suy đa cơ quan và đe dọa tính mạng. Bộ Y tế lí giải đề xuất bồi thường tai biến tiêm chủng gấp 30 lần mức lương cơ sở Cô gái trẻ suýt liệt cả 2 chân vì bỏ qua tín hiệu cảnh báo và mua thuốc tự điều trị 7 l...</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Vi rút độc lực cao đe dọa bùng phát dịch tay chân miệng ở TPHCM</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Bệnh tay chân miệng đang quay trở lại với những biểu hiện không còn điển hình khiến nhiều phụ huynh dễ chủ quan và bỏ sót dấu hiệu sớm. Sự xuất hiện của chủng virus độc lực cao Enterovirus 71 (EV 71) khiến ca bệnh tại TP.HCM tăng mạnh, ngành y tế cảnh báo nguy cơ bùng phát dịch kéo theo nhiều ca bệnh nặng ở trẻ nhỏ. Hai bệnh viện đầu ngành phối hợp mổ bóc khối u 12kg, bảo toàn cơ hội làm mẹ cho cô gái Mắc bệnh viêm mạch hiếm gặp, cô gái được chẩn đoán là viêm dạ dày Yếu tố quyết định giúp b...</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Lời khai của mắt xích quan trọng vụ 8.000 cây vàng &amp;apos;tuồn&amp;apos; từ nước ngoài vào Việt Nam</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Đỗ Minh Đức khai, dù biết là vàng lậu từ nước ngoài nhưng vẫn tiếp tay cho sai phạm do mức tiền công cao 100–150 triệu đồng/tháng.</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>irrelevant</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Tổ chức Y tế Thế giới cảnh báo nguy cơ lây lan Ebola cao tại khu vực</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Theo Tổng giám đốc WHO Tedros Adhanom Ghebreyesus, cho đến nay đã có 51 trường hợp được xác nhận ở các tỉnh Ituri và Bắc Kivu ở miền Đông Cộng hòa Dân chủ Congo. Trong khi Uganda cũng đã thông báo về 2 trường hợp nhiễm bệnh được xác nhận tại Thủ đô Kampala.</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
         <is>
           <t>relevant</t>
         </is>

</xml_diff>